<commit_message>
xlsx timestamp and col width formatting
</commit_message>
<xml_diff>
--- a/output/MONTHLY_MASTER.xlsx
+++ b/output/MONTHLY_MASTER.xlsx
@@ -17,8 +17,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -57,8 +57,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -428,101 +431,117 @@
   </sheetPr>
   <dimension ref="A1:R141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="6" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="8" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
+    <col width="19" customWidth="1" min="18" max="18"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>date</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Palm_Oil</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>FFR_midpoint</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>UST_10Y</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>VIX</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>USDMYR</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>DXY</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Brent_Oil</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>KLCI</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>cpi_inflation_yoy</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>OPR</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>MGS_10Y</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>financials</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>plantation</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>reits</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>technology</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>energy</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>industrial_products</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="2" t="n">
         <v>42035</v>
       </c>
       <c r="B2" t="n">
@@ -550,7 +569,7 @@
         <v>1781.260009765625</v>
       </c>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" s="2" t="n">
+      <c r="K2" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="L2" t="n">
@@ -574,7 +593,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" s="2" t="n">
         <v>42063</v>
       </c>
       <c r="B3" t="n">
@@ -602,7 +621,7 @@
         <v>1821.2099609375</v>
       </c>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" s="2" t="n">
+      <c r="K3" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="L3" t="n">
@@ -626,7 +645,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" s="2" t="n">
         <v>42094</v>
       </c>
       <c r="B4" t="n">
@@ -654,10 +673,10 @@
         <v>1830.780029296875</v>
       </c>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" s="2" t="n">
+      <c r="K4" s="3" t="n">
         <v>3.25</v>
       </c>
-      <c r="L4" s="2" t="n">
+      <c r="L4" s="3" t="n">
         <v>3.9</v>
       </c>
       <c r="M4" t="n">
@@ -678,7 +697,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" s="2" t="n">
         <v>42124</v>
       </c>
       <c r="B5" t="n">
@@ -706,7 +725,7 @@
         <v>1818.27001953125</v>
       </c>
       <c r="J5" t="inlineStr"/>
-      <c r="K5" s="2" t="n">
+      <c r="K5" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="L5" t="n">
@@ -730,7 +749,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" s="2" t="n">
         <v>42155</v>
       </c>
       <c r="B6" t="n">
@@ -758,7 +777,7 @@
         <v>1747.52001953125</v>
       </c>
       <c r="J6" t="inlineStr"/>
-      <c r="K6" s="2" t="n">
+      <c r="K6" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="L6" t="n">
@@ -782,7 +801,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" s="2" t="n">
         <v>42185</v>
       </c>
       <c r="B7" t="n">
@@ -810,7 +829,7 @@
         <v>1706.640014648438</v>
       </c>
       <c r="J7" t="inlineStr"/>
-      <c r="K7" s="2" t="n">
+      <c r="K7" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="L7" t="n">
@@ -834,7 +853,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" s="2" t="n">
         <v>42216</v>
       </c>
       <c r="B8" t="n">
@@ -862,7 +881,7 @@
         <v>1723.140014648438</v>
       </c>
       <c r="J8" t="inlineStr"/>
-      <c r="K8" s="2" t="n">
+      <c r="K8" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="L8" t="n">
@@ -886,7 +905,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" s="2" t="n">
         <v>42247</v>
       </c>
       <c r="B9" t="n">
@@ -910,35 +929,35 @@
       <c r="H9" t="n">
         <v>50.04999923706055</v>
       </c>
-      <c r="I9" s="2" t="n">
+      <c r="I9" s="3" t="n">
         <v>1612.739990234375</v>
       </c>
       <c r="J9" t="inlineStr"/>
-      <c r="K9" s="2" t="n">
+      <c r="K9" s="3" t="n">
         <v>3.25</v>
       </c>
-      <c r="L9" s="2" t="n">
+      <c r="L9" s="3" t="n">
         <v>4.39</v>
       </c>
-      <c r="M9" s="2" t="n">
+      <c r="M9" s="3" t="n">
         <v>97.9143571997994</v>
       </c>
       <c r="N9" t="inlineStr"/>
-      <c r="O9" s="2" t="n">
+      <c r="O9" s="3" t="n">
         <v>103.7374199862816</v>
       </c>
-      <c r="P9" s="2" t="n">
+      <c r="P9" s="3" t="n">
         <v>126.3458441526099</v>
       </c>
-      <c r="Q9" s="2" t="n">
+      <c r="Q9" s="3" t="n">
         <v>114.2937159915654</v>
       </c>
-      <c r="R9" s="2" t="n">
+      <c r="R9" s="3" t="n">
         <v>110.8244326141899</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" s="2" t="n">
         <v>42277</v>
       </c>
       <c r="B10" t="n">
@@ -966,7 +985,7 @@
         <v>1621.0400390625</v>
       </c>
       <c r="J10" t="inlineStr"/>
-      <c r="K10" s="2" t="n">
+      <c r="K10" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="L10" t="n">
@@ -990,7 +1009,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" s="2" t="n">
         <v>42308</v>
       </c>
       <c r="B11" t="n">
@@ -1018,7 +1037,7 @@
         <v>1665.7099609375</v>
       </c>
       <c r="J11" t="inlineStr"/>
-      <c r="K11" s="2" t="n">
+      <c r="K11" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="L11" t="n">
@@ -1042,7 +1061,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" s="2" t="n">
         <v>42338</v>
       </c>
       <c r="B12" t="n">
@@ -1070,7 +1089,7 @@
         <v>1672.160034179688</v>
       </c>
       <c r="J12" t="inlineStr"/>
-      <c r="K12" s="2" t="n">
+      <c r="K12" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="L12" t="n">
@@ -1094,7 +1113,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" s="2" t="n">
         <v>42369</v>
       </c>
       <c r="B13" t="n">
@@ -1122,7 +1141,7 @@
         <v>1692.510009765625</v>
       </c>
       <c r="J13" t="inlineStr"/>
-      <c r="K13" s="2" t="n">
+      <c r="K13" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="L13" t="n">
@@ -1146,7 +1165,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" s="2" t="n">
         <v>42400</v>
       </c>
       <c r="B14" t="n">
@@ -1174,7 +1193,7 @@
         <v>1667.800048828125</v>
       </c>
       <c r="J14" t="inlineStr"/>
-      <c r="K14" s="2" t="n">
+      <c r="K14" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="L14" t="n">
@@ -1198,7 +1217,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" s="2" t="n">
         <v>42429</v>
       </c>
       <c r="B15" t="n">
@@ -1226,7 +1245,7 @@
         <v>1654.75</v>
       </c>
       <c r="J15" t="inlineStr"/>
-      <c r="K15" s="2" t="n">
+      <c r="K15" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="L15" t="n">
@@ -1250,7 +1269,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" s="2" t="n">
         <v>42460</v>
       </c>
       <c r="B16" t="n">
@@ -1278,7 +1297,7 @@
         <v>1717.579956054688</v>
       </c>
       <c r="J16" t="inlineStr"/>
-      <c r="K16" s="2" t="n">
+      <c r="K16" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="L16" t="n">
@@ -1302,7 +1321,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" s="2" t="n">
         <v>42490</v>
       </c>
       <c r="B17" t="n">
@@ -1330,7 +1349,7 @@
         <v>1672.719970703125</v>
       </c>
       <c r="J17" t="inlineStr"/>
-      <c r="K17" s="2" t="n">
+      <c r="K17" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="L17" t="n">
@@ -1354,7 +1373,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" s="2" t="n">
         <v>42521</v>
       </c>
       <c r="B18" t="n">
@@ -1382,7 +1401,7 @@
         <v>1626</v>
       </c>
       <c r="J18" t="inlineStr"/>
-      <c r="K18" s="2" t="n">
+      <c r="K18" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="L18" t="n">
@@ -1406,7 +1425,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" s="2" t="n">
         <v>42551</v>
       </c>
       <c r="B19" t="n">
@@ -1434,7 +1453,7 @@
         <v>1654.079956054688</v>
       </c>
       <c r="J19" t="inlineStr"/>
-      <c r="K19" s="2" t="n">
+      <c r="K19" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="L19" t="n">
@@ -1458,7 +1477,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
+      <c r="A20" s="2" t="n">
         <v>42582</v>
       </c>
       <c r="B20" t="n">
@@ -1486,7 +1505,7 @@
         <v>1653.260009765625</v>
       </c>
       <c r="J20" t="inlineStr"/>
-      <c r="K20" s="2" t="n">
+      <c r="K20" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L20" t="n">
@@ -1510,7 +1529,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
+      <c r="A21" s="2" t="n">
         <v>42613</v>
       </c>
       <c r="B21" t="n">
@@ -1534,35 +1553,35 @@
       <c r="H21" t="n">
         <v>48.36999893188477</v>
       </c>
-      <c r="I21" s="2" t="n">
+      <c r="I21" s="3" t="n">
         <v>1678.06005859375</v>
       </c>
       <c r="J21" t="inlineStr"/>
-      <c r="K21" s="2" t="n">
+      <c r="K21" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="L21" s="2" t="n">
+      <c r="L21" s="3" t="n">
         <v>3.59</v>
       </c>
-      <c r="M21" s="2" t="n">
+      <c r="M21" s="3" t="n">
         <v>101.6910712300357</v>
       </c>
       <c r="N21" t="inlineStr"/>
-      <c r="O21" s="2" t="n">
+      <c r="O21" s="3" t="n">
         <v>125.5703385582802</v>
       </c>
-      <c r="P21" s="2" t="n">
+      <c r="P21" s="3" t="n">
         <v>160.8174323530147</v>
       </c>
-      <c r="Q21" s="2" t="n">
+      <c r="Q21" s="3" t="n">
         <v>127.4272877300538</v>
       </c>
-      <c r="R21" s="2" t="n">
+      <c r="R21" s="3" t="n">
         <v>192.8311799830827</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
+      <c r="A22" s="2" t="n">
         <v>42643</v>
       </c>
       <c r="B22" t="n">
@@ -1590,7 +1609,7 @@
         <v>1652.550048828125</v>
       </c>
       <c r="J22" t="inlineStr"/>
-      <c r="K22" s="2" t="n">
+      <c r="K22" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L22" t="n">
@@ -1614,7 +1633,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
+      <c r="A23" s="2" t="n">
         <v>42674</v>
       </c>
       <c r="B23" t="n">
@@ -1642,7 +1661,7 @@
         <v>1672.4599609375</v>
       </c>
       <c r="J23" t="inlineStr"/>
-      <c r="K23" s="2" t="n">
+      <c r="K23" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L23" t="n">
@@ -1666,7 +1685,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
+      <c r="A24" s="2" t="n">
         <v>42704</v>
       </c>
       <c r="B24" t="n">
@@ -1694,7 +1713,7 @@
         <v>1619.119995117188</v>
       </c>
       <c r="J24" t="inlineStr"/>
-      <c r="K24" s="2" t="n">
+      <c r="K24" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L24" t="n">
@@ -1718,7 +1737,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
+      <c r="A25" s="2" t="n">
         <v>42735</v>
       </c>
       <c r="B25" t="n">
@@ -1746,7 +1765,7 @@
         <v>1641.72998046875</v>
       </c>
       <c r="J25" t="inlineStr"/>
-      <c r="K25" s="2" t="n">
+      <c r="K25" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L25" t="n">
@@ -1770,7 +1789,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
+      <c r="A26" s="2" t="n">
         <v>42766</v>
       </c>
       <c r="B26" t="n">
@@ -1798,7 +1817,7 @@
         <v>1671.5400390625</v>
       </c>
       <c r="J26" t="inlineStr"/>
-      <c r="K26" s="2" t="n">
+      <c r="K26" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L26" t="n">
@@ -1822,7 +1841,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
+      <c r="A27" s="2" t="n">
         <v>42794</v>
       </c>
       <c r="B27" t="n">
@@ -1850,7 +1869,7 @@
         <v>1693.77001953125</v>
       </c>
       <c r="J27" t="inlineStr"/>
-      <c r="K27" s="2" t="n">
+      <c r="K27" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L27" t="n">
@@ -1874,7 +1893,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
+      <c r="A28" s="2" t="n">
         <v>42825</v>
       </c>
       <c r="B28" t="n">
@@ -1902,7 +1921,7 @@
         <v>1740.089965820312</v>
       </c>
       <c r="J28" t="inlineStr"/>
-      <c r="K28" s="2" t="n">
+      <c r="K28" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L28" t="n">
@@ -1926,7 +1945,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
+      <c r="A29" s="2" t="n">
         <v>42855</v>
       </c>
       <c r="B29" t="n">
@@ -1954,7 +1973,7 @@
         <v>1768.06005859375</v>
       </c>
       <c r="J29" t="inlineStr"/>
-      <c r="K29" s="2" t="n">
+      <c r="K29" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L29" t="n">
@@ -1978,7 +1997,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
+      <c r="A30" s="2" t="n">
         <v>42886</v>
       </c>
       <c r="B30" t="n">
@@ -2006,7 +2025,7 @@
         <v>1765.869995117188</v>
       </c>
       <c r="J30" t="inlineStr"/>
-      <c r="K30" s="2" t="n">
+      <c r="K30" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L30" t="n">
@@ -2030,7 +2049,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
+      <c r="A31" s="2" t="n">
         <v>42916</v>
       </c>
       <c r="B31" t="n">
@@ -2058,7 +2077,7 @@
         <v>1763.670043945312</v>
       </c>
       <c r="J31" t="inlineStr"/>
-      <c r="K31" s="2" t="n">
+      <c r="K31" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L31" t="n">
@@ -2082,7 +2101,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="n">
+      <c r="A32" s="2" t="n">
         <v>42947</v>
       </c>
       <c r="B32" t="n">
@@ -2110,7 +2129,7 @@
         <v>1760.030029296875</v>
       </c>
       <c r="J32" t="inlineStr"/>
-      <c r="K32" s="2" t="n">
+      <c r="K32" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L32" t="n">
@@ -2134,7 +2153,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
+      <c r="A33" s="2" t="n">
         <v>42978</v>
       </c>
       <c r="B33" t="n">
@@ -2158,14 +2177,14 @@
       <c r="H33" t="n">
         <v>50.86000061035156</v>
       </c>
-      <c r="I33" s="2" t="n">
+      <c r="I33" s="3" t="n">
         <v>1773.160034179688</v>
       </c>
       <c r="J33" t="inlineStr"/>
-      <c r="K33" s="2" t="n">
+      <c r="K33" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="L33" s="2" t="n">
+      <c r="L33" s="3" t="n">
         <v>3.89</v>
       </c>
       <c r="M33" t="n">
@@ -2186,7 +2205,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
+      <c r="A34" s="2" t="n">
         <v>43008</v>
       </c>
       <c r="B34" t="n">
@@ -2214,7 +2233,7 @@
         <v>1755.579956054688</v>
       </c>
       <c r="J34" t="inlineStr"/>
-      <c r="K34" s="2" t="n">
+      <c r="K34" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L34" t="n">
@@ -2238,7 +2257,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
+      <c r="A35" s="2" t="n">
         <v>43039</v>
       </c>
       <c r="B35" t="n">
@@ -2266,7 +2285,7 @@
         <v>1747.920043945312</v>
       </c>
       <c r="J35" t="inlineStr"/>
-      <c r="K35" s="2" t="n">
+      <c r="K35" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L35" t="n">
@@ -2290,7 +2309,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
+      <c r="A36" s="2" t="n">
         <v>43069</v>
       </c>
       <c r="B36" t="n">
@@ -2318,7 +2337,7 @@
         <v>1717.859985351562</v>
       </c>
       <c r="J36" t="inlineStr"/>
-      <c r="K36" s="2" t="n">
+      <c r="K36" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L36" t="n">
@@ -2344,7 +2363,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
+      <c r="A37" s="2" t="n">
         <v>43100</v>
       </c>
       <c r="B37" t="n">
@@ -2372,7 +2391,7 @@
         <v>1796.81005859375</v>
       </c>
       <c r="J37" t="inlineStr"/>
-      <c r="K37" s="2" t="n">
+      <c r="K37" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L37" t="n">
@@ -2398,7 +2417,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
+      <c r="A38" s="2" t="n">
         <v>43131</v>
       </c>
       <c r="B38" t="n">
@@ -2422,37 +2441,37 @@
       <c r="H38" t="n">
         <v>69.01999664306641</v>
       </c>
-      <c r="I38" s="2" t="n">
+      <c r="I38" s="3" t="n">
         <v>1868.579956054688</v>
       </c>
       <c r="J38" t="inlineStr"/>
-      <c r="K38" s="2" t="n">
+      <c r="K38" s="3" t="n">
         <v>3.25</v>
       </c>
-      <c r="L38" s="2" t="n">
+      <c r="L38" s="3" t="n">
         <v>3.96</v>
       </c>
-      <c r="M38" s="2" t="n">
+      <c r="M38" s="3" t="n">
         <v>139.2056070289008</v>
       </c>
-      <c r="N38" s="2" t="n">
+      <c r="N38" s="3" t="n">
         <v>106.3690987258629</v>
       </c>
-      <c r="O38" s="2" t="n">
+      <c r="O38" s="3" t="n">
         <v>131.3477012859881</v>
       </c>
-      <c r="P38" s="2" t="n">
+      <c r="P38" s="3" t="n">
         <v>481.752107018418</v>
       </c>
-      <c r="Q38" s="2" t="n">
+      <c r="Q38" s="3" t="n">
         <v>135.6503114629042</v>
       </c>
-      <c r="R38" s="2" t="n">
+      <c r="R38" s="3" t="n">
         <v>594.7357734359055</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
+      <c r="A39" s="2" t="n">
         <v>43159</v>
       </c>
       <c r="B39" t="n">
@@ -2480,7 +2499,7 @@
         <v>1856.199951171875</v>
       </c>
       <c r="J39" t="inlineStr"/>
-      <c r="K39" s="2" t="n">
+      <c r="K39" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="L39" t="n">
@@ -2506,7 +2525,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
+      <c r="A40" s="2" t="n">
         <v>43190</v>
       </c>
       <c r="B40" t="n">
@@ -2515,26 +2534,26 @@
       <c r="C40" t="n">
         <v>1.625</v>
       </c>
-      <c r="D40" s="2" t="n">
+      <c r="D40" s="3" t="n">
         <v>2.740999937057495</v>
       </c>
-      <c r="E40" s="2" t="n">
+      <c r="E40" s="3" t="n">
         <v>19.96999931335449</v>
       </c>
       <c r="F40" t="n">
         <v>3.865000009536743</v>
       </c>
-      <c r="G40" s="2" t="n">
+      <c r="G40" s="3" t="n">
         <v>90.15000152587891</v>
       </c>
-      <c r="H40" s="2" t="n">
+      <c r="H40" s="3" t="n">
         <v>70.26999664306641</v>
       </c>
       <c r="I40" t="n">
         <v>1863.4599609375</v>
       </c>
       <c r="J40" t="inlineStr"/>
-      <c r="K40" s="2" t="n">
+      <c r="K40" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="L40" t="n">
@@ -2560,7 +2579,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
+      <c r="A41" s="2" t="n">
         <v>43220</v>
       </c>
       <c r="B41" t="n">
@@ -2588,7 +2607,7 @@
         <v>1870.369995117188</v>
       </c>
       <c r="J41" t="inlineStr"/>
-      <c r="K41" s="2" t="n">
+      <c r="K41" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="L41" t="n">
@@ -2614,7 +2633,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="n">
+      <c r="A42" s="2" t="n">
         <v>43251</v>
       </c>
       <c r="B42" t="n">
@@ -2642,7 +2661,7 @@
         <v>1740.619995117188</v>
       </c>
       <c r="J42" t="inlineStr"/>
-      <c r="K42" s="2" t="n">
+      <c r="K42" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="L42" t="n">
@@ -2668,7 +2687,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n">
+      <c r="A43" s="2" t="n">
         <v>43281</v>
       </c>
       <c r="B43" t="n">
@@ -2696,7 +2715,7 @@
         <v>1691.5</v>
       </c>
       <c r="J43" t="inlineStr"/>
-      <c r="K43" s="2" t="n">
+      <c r="K43" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="L43" t="n">
@@ -2722,7 +2741,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
+      <c r="A44" s="2" t="n">
         <v>43312</v>
       </c>
       <c r="B44" t="n">
@@ -2750,7 +2769,7 @@
         <v>1784.25</v>
       </c>
       <c r="J44" t="inlineStr"/>
-      <c r="K44" s="2" t="n">
+      <c r="K44" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="L44" t="n">
@@ -2776,7 +2795,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
+      <c r="A45" s="2" t="n">
         <v>43343</v>
       </c>
       <c r="B45" t="n">
@@ -2800,37 +2819,37 @@
       <c r="H45" t="n">
         <v>77.76999664306641</v>
       </c>
-      <c r="I45" s="2" t="n">
+      <c r="I45" s="3" t="n">
         <v>1819.660034179688</v>
       </c>
       <c r="J45" t="inlineStr"/>
-      <c r="K45" s="2" t="n">
+      <c r="K45" s="3" t="n">
         <v>3.25</v>
       </c>
-      <c r="L45" s="2" t="n">
+      <c r="L45" s="3" t="n">
         <v>4.04</v>
       </c>
-      <c r="M45" s="2" t="n">
+      <c r="M45" s="3" t="n">
         <v>140.3911315882537</v>
       </c>
-      <c r="N45" s="2" t="n">
+      <c r="N45" s="3" t="n">
         <v>105.374234555994</v>
       </c>
-      <c r="O45" s="2" t="n">
+      <c r="O45" s="3" t="n">
         <v>141.4153321382273</v>
       </c>
-      <c r="P45" s="2" t="n">
+      <c r="P45" s="3" t="n">
         <v>662.7670105801706</v>
       </c>
-      <c r="Q45" s="2" t="n">
+      <c r="Q45" s="3" t="n">
         <v>154.9234626415269</v>
       </c>
-      <c r="R45" s="2" t="n">
+      <c r="R45" s="3" t="n">
         <v>625.4760320899331</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
+      <c r="A46" s="2" t="n">
         <v>43373</v>
       </c>
       <c r="B46" t="n">
@@ -2858,7 +2877,7 @@
         <v>1793.150024414062</v>
       </c>
       <c r="J46" t="inlineStr"/>
-      <c r="K46" s="2" t="n">
+      <c r="K46" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="L46" t="n">
@@ -2884,7 +2903,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
+      <c r="A47" s="2" t="n">
         <v>43404</v>
       </c>
       <c r="B47" t="n">
@@ -2912,7 +2931,7 @@
         <v>1709.27001953125</v>
       </c>
       <c r="J47" t="inlineStr"/>
-      <c r="K47" s="2" t="n">
+      <c r="K47" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="L47" t="n">
@@ -2938,7 +2957,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
+      <c r="A48" s="2" t="n">
         <v>43434</v>
       </c>
       <c r="B48" t="n">
@@ -2966,7 +2985,7 @@
         <v>1679.859985351562</v>
       </c>
       <c r="J48" t="inlineStr"/>
-      <c r="K48" s="2" t="n">
+      <c r="K48" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="L48" t="n">
@@ -2992,7 +3011,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1" t="n">
+      <c r="A49" s="2" t="n">
         <v>43465</v>
       </c>
       <c r="B49" t="n">
@@ -3020,7 +3039,7 @@
         <v>1690.579956054688</v>
       </c>
       <c r="J49" t="inlineStr"/>
-      <c r="K49" s="2" t="n">
+      <c r="K49" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="L49" t="n">
@@ -3046,7 +3065,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="n">
+      <c r="A50" s="2" t="n">
         <v>43496</v>
       </c>
       <c r="B50" t="n">
@@ -3074,7 +3093,7 @@
         <v>1683.530029296875</v>
       </c>
       <c r="J50" t="inlineStr"/>
-      <c r="K50" s="2" t="n">
+      <c r="K50" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="L50" t="n">
@@ -3100,7 +3119,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="n">
+      <c r="A51" s="2" t="n">
         <v>43524</v>
       </c>
       <c r="B51" t="n">
@@ -3130,7 +3149,7 @@
       <c r="J51" t="n">
         <v>0.2</v>
       </c>
-      <c r="K51" s="2" t="n">
+      <c r="K51" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="L51" t="n">
@@ -3156,7 +3175,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="n">
+      <c r="A52" s="2" t="n">
         <v>43555</v>
       </c>
       <c r="B52" t="n">
@@ -3186,7 +3205,7 @@
       <c r="J52" t="n">
         <v>0.3</v>
       </c>
-      <c r="K52" s="2" t="n">
+      <c r="K52" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="L52" t="n">
@@ -3212,7 +3231,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="n">
+      <c r="A53" s="2" t="n">
         <v>43585</v>
       </c>
       <c r="B53" t="n">
@@ -3242,7 +3261,7 @@
       <c r="J53" t="n">
         <v>0.5</v>
       </c>
-      <c r="K53" s="2" t="n">
+      <c r="K53" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="L53" t="n">
@@ -3268,7 +3287,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="n">
+      <c r="A54" s="2" t="n">
         <v>43616</v>
       </c>
       <c r="B54" t="n">
@@ -3298,7 +3317,7 @@
       <c r="J54" t="n">
         <v>0.5</v>
       </c>
-      <c r="K54" s="2" t="n">
+      <c r="K54" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L54" t="n">
@@ -3324,7 +3343,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="n">
+      <c r="A55" s="2" t="n">
         <v>43646</v>
       </c>
       <c r="B55" t="n">
@@ -3354,7 +3373,7 @@
       <c r="J55" t="n">
         <v>0.4</v>
       </c>
-      <c r="K55" s="2" t="n">
+      <c r="K55" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L55" t="n">
@@ -3380,7 +3399,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="1" t="n">
+      <c r="A56" s="2" t="n">
         <v>43677</v>
       </c>
       <c r="B56" t="n">
@@ -3410,7 +3429,7 @@
       <c r="J56" t="n">
         <v>1.9</v>
       </c>
-      <c r="K56" s="2" t="n">
+      <c r="K56" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L56" t="n">
@@ -3436,7 +3455,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="1" t="n">
+      <c r="A57" s="2" t="n">
         <v>43708</v>
       </c>
       <c r="B57" t="n">
@@ -3466,7 +3485,7 @@
       <c r="J57" t="n">
         <v>2</v>
       </c>
-      <c r="K57" s="2" t="n">
+      <c r="K57" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L57" t="n">
@@ -3492,7 +3511,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="1" t="n">
+      <c r="A58" s="2" t="n">
         <v>43738</v>
       </c>
       <c r="B58" t="n">
@@ -3522,7 +3541,7 @@
       <c r="J58" t="n">
         <v>2</v>
       </c>
-      <c r="K58" s="2" t="n">
+      <c r="K58" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L58" t="n">
@@ -3548,7 +3567,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="1" t="n">
+      <c r="A59" s="2" t="n">
         <v>43769</v>
       </c>
       <c r="B59" t="n">
@@ -3578,7 +3597,7 @@
       <c r="J59" t="n">
         <v>1.5</v>
       </c>
-      <c r="K59" s="2" t="n">
+      <c r="K59" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L59" t="n">
@@ -3604,7 +3623,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="1" t="n">
+      <c r="A60" s="2" t="n">
         <v>43799</v>
       </c>
       <c r="B60" t="n">
@@ -3634,7 +3653,7 @@
       <c r="J60" t="n">
         <v>1.4</v>
       </c>
-      <c r="K60" s="2" t="n">
+      <c r="K60" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L60" t="n">
@@ -3660,7 +3679,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="1" t="n">
+      <c r="A61" s="2" t="n">
         <v>43830</v>
       </c>
       <c r="B61" t="n">
@@ -3690,7 +3709,7 @@
       <c r="J61" t="n">
         <v>1.4</v>
       </c>
-      <c r="K61" s="2" t="n">
+      <c r="K61" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L61" t="n">
@@ -3716,7 +3735,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="1" t="n">
+      <c r="A62" s="2" t="n">
         <v>43861</v>
       </c>
       <c r="B62" t="n">
@@ -3746,7 +3765,7 @@
       <c r="J62" t="n">
         <v>1.4</v>
       </c>
-      <c r="K62" s="2" t="n">
+      <c r="K62" s="3" t="n">
         <v>2.75</v>
       </c>
       <c r="L62" t="n">
@@ -3772,7 +3791,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="1" t="n">
+      <c r="A63" s="2" t="n">
         <v>43890</v>
       </c>
       <c r="B63" t="n">
@@ -3802,7 +3821,7 @@
       <c r="J63" t="n">
         <v>1.6</v>
       </c>
-      <c r="K63" s="2" t="n">
+      <c r="K63" s="3" t="n">
         <v>2.75</v>
       </c>
       <c r="L63" t="n">
@@ -3828,7 +3847,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="1" t="n">
+      <c r="A64" s="2" t="n">
         <v>43921</v>
       </c>
       <c r="B64" t="n">
@@ -3858,7 +3877,7 @@
       <c r="J64" t="n">
         <v>1.3</v>
       </c>
-      <c r="K64" s="2" t="n">
+      <c r="K64" s="3" t="n">
         <v>2.5</v>
       </c>
       <c r="L64" t="n">
@@ -3884,7 +3903,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="1" t="n">
+      <c r="A65" s="2" t="n">
         <v>43951</v>
       </c>
       <c r="B65" t="n">
@@ -3914,7 +3933,7 @@
       <c r="J65" t="n">
         <v>1.3</v>
       </c>
-      <c r="K65" s="2" t="n">
+      <c r="K65" s="3" t="n">
         <v>2.5</v>
       </c>
       <c r="L65" t="n">
@@ -3940,7 +3959,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="1" t="n">
+      <c r="A66" s="2" t="n">
         <v>43982</v>
       </c>
       <c r="B66" t="n">
@@ -3970,7 +3989,7 @@
       <c r="J66" t="n">
         <v>1.3</v>
       </c>
-      <c r="K66" s="2" t="n">
+      <c r="K66" s="3" t="n">
         <v>2</v>
       </c>
       <c r="L66" t="n">
@@ -3996,7 +4015,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="1" t="n">
+      <c r="A67" s="2" t="n">
         <v>44012</v>
       </c>
       <c r="B67" t="n">
@@ -4026,7 +4045,7 @@
       <c r="J67" t="n">
         <v>1.1</v>
       </c>
-      <c r="K67" s="2" t="n">
+      <c r="K67" s="3" t="n">
         <v>2</v>
       </c>
       <c r="L67" t="n">
@@ -4052,7 +4071,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="1" t="n">
+      <c r="A68" s="2" t="n">
         <v>44043</v>
       </c>
       <c r="B68" t="n">
@@ -4076,39 +4095,39 @@
       <c r="H68" t="n">
         <v>42.93999862670898</v>
       </c>
-      <c r="I68" s="2" t="n">
+      <c r="I68" s="3" t="n">
         <v>1603.75</v>
       </c>
       <c r="J68" t="n">
         <v>1.2</v>
       </c>
-      <c r="K68" s="2" t="n">
+      <c r="K68" s="3" t="n">
         <v>1.75</v>
       </c>
-      <c r="L68" s="2" t="n">
+      <c r="L68" s="3" t="n">
         <v>2.55</v>
       </c>
-      <c r="M68" s="2" t="n">
+      <c r="M68" s="3" t="n">
         <v>106.5134710375964</v>
       </c>
-      <c r="N68" s="2" t="n">
+      <c r="N68" s="3" t="n">
         <v>109.4835644868736</v>
       </c>
-      <c r="O68" s="2" t="n">
+      <c r="O68" s="3" t="n">
         <v>154.0140903824953</v>
       </c>
-      <c r="P68" s="2" t="n">
+      <c r="P68" s="3" t="n">
         <v>1369.519696446954</v>
       </c>
-      <c r="Q68" s="2" t="n">
+      <c r="Q68" s="3" t="n">
         <v>132.9471918091454</v>
       </c>
-      <c r="R68" s="2" t="n">
+      <c r="R68" s="3" t="n">
         <v>1437.456952473097</v>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="1" t="n">
+      <c r="A69" s="2" t="n">
         <v>44074</v>
       </c>
       <c r="B69" t="n">
@@ -4132,39 +4151,39 @@
       <c r="H69" t="n">
         <v>45.04999923706055</v>
       </c>
-      <c r="I69" s="2" t="n">
+      <c r="I69" s="3" t="n">
         <v>1525.2099609375</v>
       </c>
       <c r="J69" t="n">
         <v>1.1</v>
       </c>
-      <c r="K69" s="2" t="n">
+      <c r="K69" s="3" t="n">
         <v>1.75</v>
       </c>
-      <c r="L69" s="2" t="n">
+      <c r="L69" s="3" t="n">
         <v>2.6</v>
       </c>
-      <c r="M69" s="2" t="n">
+      <c r="M69" s="3" t="n">
         <v>100.8568794478521</v>
       </c>
-      <c r="N69" s="2" t="n">
+      <c r="N69" s="3" t="n">
         <v>106.644249630433</v>
       </c>
-      <c r="O69" s="2" t="n">
+      <c r="O69" s="3" t="n">
         <v>157.8706633056499</v>
       </c>
-      <c r="P69" s="2" t="n">
+      <c r="P69" s="3" t="n">
         <v>1432.372003574803</v>
       </c>
-      <c r="Q69" s="2" t="n">
+      <c r="Q69" s="3" t="n">
         <v>125.1881324044122</v>
       </c>
-      <c r="R69" s="2" t="n">
+      <c r="R69" s="3" t="n">
         <v>1518.658006783828</v>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="1" t="n">
+      <c r="A70" s="2" t="n">
         <v>44104</v>
       </c>
       <c r="B70" t="n">
@@ -4194,7 +4213,7 @@
       <c r="J70" t="n">
         <v>1.1</v>
       </c>
-      <c r="K70" s="2" t="n">
+      <c r="K70" s="3" t="n">
         <v>1.75</v>
       </c>
       <c r="L70" t="n">
@@ -4220,7 +4239,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="1" t="n">
+      <c r="A71" s="2" t="n">
         <v>44135</v>
       </c>
       <c r="B71" t="n">
@@ -4250,7 +4269,7 @@
       <c r="J71" t="n">
         <v>1</v>
       </c>
-      <c r="K71" s="2" t="n">
+      <c r="K71" s="3" t="n">
         <v>1.75</v>
       </c>
       <c r="L71" t="n">
@@ -4276,7 +4295,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="1" t="n">
+      <c r="A72" s="2" t="n">
         <v>44165</v>
       </c>
       <c r="B72" t="n">
@@ -4306,7 +4325,7 @@
       <c r="J72" t="n">
         <v>0.8</v>
       </c>
-      <c r="K72" s="2" t="n">
+      <c r="K72" s="3" t="n">
         <v>1.75</v>
       </c>
       <c r="L72" t="n">
@@ -4332,7 +4351,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="1" t="n">
+      <c r="A73" s="2" t="n">
         <v>44196</v>
       </c>
       <c r="B73" t="n">
@@ -4362,7 +4381,7 @@
       <c r="J73" t="n">
         <v>0.7</v>
       </c>
-      <c r="K73" s="2" t="n">
+      <c r="K73" s="3" t="n">
         <v>1.75</v>
       </c>
       <c r="L73" t="n">
@@ -4388,7 +4407,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="1" t="n">
+      <c r="A74" s="2" t="n">
         <v>44227</v>
       </c>
       <c r="B74" t="n">
@@ -4418,7 +4437,7 @@
       <c r="J74" t="n">
         <v>0.7</v>
       </c>
-      <c r="K74" s="2" t="n">
+      <c r="K74" s="3" t="n">
         <v>1.75</v>
       </c>
       <c r="L74" t="n">
@@ -4444,7 +4463,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="1" t="n">
+      <c r="A75" s="2" t="n">
         <v>44255</v>
       </c>
       <c r="B75" t="n">
@@ -4474,7 +4493,7 @@
       <c r="J75" t="n">
         <v>0.7</v>
       </c>
-      <c r="K75" s="2" t="n">
+      <c r="K75" s="3" t="n">
         <v>1.75</v>
       </c>
       <c r="L75" t="n">
@@ -4500,7 +4519,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="1" t="n">
+      <c r="A76" s="2" t="n">
         <v>44286</v>
       </c>
       <c r="B76" t="n">
@@ -4530,7 +4549,7 @@
       <c r="J76" t="n">
         <v>0.7</v>
       </c>
-      <c r="K76" s="2" t="n">
+      <c r="K76" s="3" t="n">
         <v>1.75</v>
       </c>
       <c r="L76" t="n">
@@ -4556,7 +4575,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="1" t="n">
+      <c r="A77" s="2" t="n">
         <v>44316</v>
       </c>
       <c r="B77" t="n">
@@ -4586,7 +4605,7 @@
       <c r="J77" t="n">
         <v>0.7</v>
       </c>
-      <c r="K77" s="2" t="n">
+      <c r="K77" s="3" t="n">
         <v>1.75</v>
       </c>
       <c r="L77" t="n">
@@ -4612,7 +4631,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="1" t="n">
+      <c r="A78" s="2" t="n">
         <v>44347</v>
       </c>
       <c r="B78" t="n">
@@ -4621,19 +4640,19 @@
       <c r="C78" t="n">
         <v>0.125</v>
       </c>
-      <c r="D78" s="2" t="n">
+      <c r="D78" s="3" t="n">
         <v>1.580999970436096</v>
       </c>
-      <c r="E78" s="2" t="n">
+      <c r="E78" s="3" t="n">
         <v>16.76000022888184</v>
       </c>
       <c r="F78" t="n">
         <v>4.13700008392334</v>
       </c>
-      <c r="G78" s="2" t="n">
+      <c r="G78" s="3" t="n">
         <v>90.02999877929688</v>
       </c>
-      <c r="H78" s="2" t="n">
+      <c r="H78" s="3" t="n">
         <v>69.62999725341797</v>
       </c>
       <c r="I78" t="n">
@@ -4642,7 +4661,7 @@
       <c r="J78" t="n">
         <v>0.7</v>
       </c>
-      <c r="K78" s="2" t="n">
+      <c r="K78" s="3" t="n">
         <v>1.75</v>
       </c>
       <c r="L78" t="n">
@@ -4668,7 +4687,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="1" t="n">
+      <c r="A79" s="2" t="n">
         <v>44377</v>
       </c>
       <c r="B79" t="n">
@@ -4698,7 +4717,7 @@
       <c r="J79" t="n">
         <v>0.8</v>
       </c>
-      <c r="K79" s="2" t="n">
+      <c r="K79" s="3" t="n">
         <v>1.75</v>
       </c>
       <c r="L79" t="n">
@@ -4724,7 +4743,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="1" t="n">
+      <c r="A80" s="2" t="n">
         <v>44408</v>
       </c>
       <c r="B80" t="n">
@@ -4754,7 +4773,7 @@
       <c r="J80" t="n">
         <v>0.7</v>
       </c>
-      <c r="K80" s="2" t="n">
+      <c r="K80" s="3" t="n">
         <v>1.75</v>
       </c>
       <c r="L80" t="n">
@@ -4780,7 +4799,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="1" t="n">
+      <c r="A81" s="2" t="n">
         <v>44439</v>
       </c>
       <c r="B81" t="n">
@@ -4804,39 +4823,39 @@
       <c r="H81" t="n">
         <v>73.41000366210938</v>
       </c>
-      <c r="I81" s="2" t="n">
+      <c r="I81" s="3" t="n">
         <v>1601.380004882812</v>
       </c>
       <c r="J81" t="n">
         <v>0.7</v>
       </c>
-      <c r="K81" s="2" t="n">
+      <c r="K81" s="3" t="n">
         <v>1.75</v>
       </c>
-      <c r="L81" s="2" t="n">
+      <c r="L81" s="3" t="n">
         <v>3.19</v>
       </c>
-      <c r="M81" s="2" t="n">
+      <c r="M81" s="3" t="n">
         <v>136.0921932443209</v>
       </c>
-      <c r="N81" s="2" t="n">
+      <c r="N81" s="3" t="n">
         <v>97.41067025957099</v>
       </c>
-      <c r="O81" s="2" t="n">
+      <c r="O81" s="3" t="n">
         <v>147.1370343027404</v>
       </c>
-      <c r="P81" s="2" t="n">
+      <c r="P81" s="3" t="n">
         <v>2199.752249890296</v>
       </c>
-      <c r="Q81" s="2" t="n">
+      <c r="Q81" s="3" t="n">
         <v>152.0642289470919</v>
       </c>
-      <c r="R81" s="2" t="n">
+      <c r="R81" s="3" t="n">
         <v>1649.043784975109</v>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="1" t="n">
+      <c r="A82" s="2" t="n">
         <v>44469</v>
       </c>
       <c r="B82" t="n">
@@ -4866,7 +4885,7 @@
       <c r="J82" t="n">
         <v>0.6</v>
       </c>
-      <c r="K82" s="2" t="n">
+      <c r="K82" s="3" t="n">
         <v>1.75</v>
       </c>
       <c r="L82" t="n">
@@ -4892,7 +4911,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="1" t="n">
+      <c r="A83" s="2" t="n">
         <v>44500</v>
       </c>
       <c r="B83" t="n">
@@ -4922,7 +4941,7 @@
       <c r="J83" t="n">
         <v>0.6</v>
       </c>
-      <c r="K83" s="2" t="n">
+      <c r="K83" s="3" t="n">
         <v>1.75</v>
       </c>
       <c r="L83" t="n">
@@ -4948,7 +4967,7 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="1" t="n">
+      <c r="A84" s="2" t="n">
         <v>44530</v>
       </c>
       <c r="B84" t="n">
@@ -4978,7 +4997,7 @@
       <c r="J84" t="n">
         <v>0.7</v>
       </c>
-      <c r="K84" s="2" t="n">
+      <c r="K84" s="3" t="n">
         <v>1.75</v>
       </c>
       <c r="L84" t="n">
@@ -5004,7 +5023,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="1" t="n">
+      <c r="A85" s="2" t="n">
         <v>44561</v>
       </c>
       <c r="B85" t="n">
@@ -5034,7 +5053,7 @@
       <c r="J85" t="n">
         <v>0.9</v>
       </c>
-      <c r="K85" s="2" t="n">
+      <c r="K85" s="3" t="n">
         <v>1.75</v>
       </c>
       <c r="L85" t="n">
@@ -5060,7 +5079,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="1" t="n">
+      <c r="A86" s="2" t="n">
         <v>44592</v>
       </c>
       <c r="B86" t="n">
@@ -5090,7 +5109,7 @@
       <c r="J86" t="n">
         <v>1.1</v>
       </c>
-      <c r="K86" s="2" t="n">
+      <c r="K86" s="3" t="n">
         <v>1.75</v>
       </c>
       <c r="L86" t="n">
@@ -5116,7 +5135,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="1" t="n">
+      <c r="A87" s="2" t="n">
         <v>44620</v>
       </c>
       <c r="B87" t="n">
@@ -5146,7 +5165,7 @@
       <c r="J87" t="n">
         <v>1.6</v>
       </c>
-      <c r="K87" s="2" t="n">
+      <c r="K87" s="3" t="n">
         <v>1.75</v>
       </c>
       <c r="L87" t="n">
@@ -5172,7 +5191,7 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="1" t="n">
+      <c r="A88" s="2" t="n">
         <v>44651</v>
       </c>
       <c r="B88" t="n">
@@ -5202,7 +5221,7 @@
       <c r="J88" t="n">
         <v>1.8</v>
       </c>
-      <c r="K88" s="2" t="n">
+      <c r="K88" s="3" t="n">
         <v>1.75</v>
       </c>
       <c r="L88" t="n">
@@ -5228,7 +5247,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="1" t="n">
+      <c r="A89" s="2" t="n">
         <v>44681</v>
       </c>
       <c r="B89" t="n">
@@ -5258,7 +5277,7 @@
       <c r="J89" t="n">
         <v>2</v>
       </c>
-      <c r="K89" s="2" t="n">
+      <c r="K89" s="3" t="n">
         <v>1.75</v>
       </c>
       <c r="L89" t="n">
@@ -5284,7 +5303,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="1" t="n">
+      <c r="A90" s="2" t="n">
         <v>44712</v>
       </c>
       <c r="B90" t="n">
@@ -5314,7 +5333,7 @@
       <c r="J90" t="n">
         <v>2.1</v>
       </c>
-      <c r="K90" s="2" t="n">
+      <c r="K90" s="3" t="n">
         <v>2</v>
       </c>
       <c r="L90" t="n">
@@ -5340,7 +5359,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="1" t="n">
+      <c r="A91" s="2" t="n">
         <v>44742</v>
       </c>
       <c r="B91" t="n">
@@ -5370,7 +5389,7 @@
       <c r="J91" t="n">
         <v>2.4</v>
       </c>
-      <c r="K91" s="2" t="n">
+      <c r="K91" s="3" t="n">
         <v>2</v>
       </c>
       <c r="L91" t="n">
@@ -5396,7 +5415,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="1" t="n">
+      <c r="A92" s="2" t="n">
         <v>44773</v>
       </c>
       <c r="B92" t="n">
@@ -5426,7 +5445,7 @@
       <c r="J92" t="n">
         <v>3</v>
       </c>
-      <c r="K92" s="2" t="n">
+      <c r="K92" s="3" t="n">
         <v>2.25</v>
       </c>
       <c r="L92" t="n">
@@ -5452,7 +5471,7 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="1" t="n">
+      <c r="A93" s="2" t="n">
         <v>44804</v>
       </c>
       <c r="B93" t="n">
@@ -5476,39 +5495,39 @@
       <c r="H93" t="n">
         <v>99.30999755859375</v>
       </c>
-      <c r="I93" s="2" t="n">
+      <c r="I93" s="3" t="n">
         <v>1512.050048828125</v>
       </c>
       <c r="J93" t="n">
         <v>3.4</v>
       </c>
-      <c r="K93" s="2" t="n">
+      <c r="K93" s="3" t="n">
         <v>2.25</v>
       </c>
-      <c r="L93" s="2" t="n">
+      <c r="L93" s="3" t="n">
         <v>3.98</v>
       </c>
-      <c r="M93" s="2" t="n">
+      <c r="M93" s="3" t="n">
         <v>157.4945593653339</v>
       </c>
-      <c r="N93" s="2" t="n">
+      <c r="N93" s="3" t="n">
         <v>110.1823738316121</v>
       </c>
-      <c r="O93" s="2" t="n">
+      <c r="O93" s="3" t="n">
         <v>155.7363442381577</v>
       </c>
-      <c r="P93" s="2" t="n">
+      <c r="P93" s="3" t="n">
         <v>1814.667077260901</v>
       </c>
-      <c r="Q93" s="2" t="n">
+      <c r="Q93" s="3" t="n">
         <v>175.9636848882157</v>
       </c>
-      <c r="R93" s="2" t="n">
+      <c r="R93" s="3" t="n">
         <v>751.7745839516789</v>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="1" t="n">
+      <c r="A94" s="2" t="n">
         <v>44834</v>
       </c>
       <c r="B94" t="n">
@@ -5538,7 +5557,7 @@
       <c r="J94" t="n">
         <v>3.8</v>
       </c>
-      <c r="K94" s="2" t="n">
+      <c r="K94" s="3" t="n">
         <v>2.5</v>
       </c>
       <c r="L94" t="n">
@@ -5564,7 +5583,7 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="1" t="n">
+      <c r="A95" s="2" t="n">
         <v>44865</v>
       </c>
       <c r="B95" t="n">
@@ -5594,7 +5613,7 @@
       <c r="J95" t="n">
         <v>4</v>
       </c>
-      <c r="K95" s="2" t="n">
+      <c r="K95" s="3" t="n">
         <v>2.5</v>
       </c>
       <c r="L95" t="n">
@@ -5620,7 +5639,7 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="1" t="n">
+      <c r="A96" s="2" t="n">
         <v>44895</v>
       </c>
       <c r="B96" t="n">
@@ -5650,7 +5669,7 @@
       <c r="J96" t="n">
         <v>4.1</v>
       </c>
-      <c r="K96" s="2" t="n">
+      <c r="K96" s="3" t="n">
         <v>2.75</v>
       </c>
       <c r="L96" t="n">
@@ -5676,7 +5695,7 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="1" t="n">
+      <c r="A97" s="2" t="n">
         <v>44926</v>
       </c>
       <c r="B97" t="n">
@@ -5706,7 +5725,7 @@
       <c r="J97" t="n">
         <v>4.2</v>
       </c>
-      <c r="K97" s="2" t="n">
+      <c r="K97" s="3" t="n">
         <v>2.75</v>
       </c>
       <c r="L97" t="n">
@@ -5732,7 +5751,7 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="1" t="n">
+      <c r="A98" s="2" t="n">
         <v>44957</v>
       </c>
       <c r="B98" t="n">
@@ -5762,7 +5781,7 @@
       <c r="J98" t="n">
         <v>4.1</v>
       </c>
-      <c r="K98" s="2" t="n">
+      <c r="K98" s="3" t="n">
         <v>2.75</v>
       </c>
       <c r="L98" t="n">
@@ -5788,7 +5807,7 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="1" t="n">
+      <c r="A99" s="2" t="n">
         <v>44985</v>
       </c>
       <c r="B99" t="n">
@@ -5818,7 +5837,7 @@
       <c r="J99" t="n">
         <v>3.9</v>
       </c>
-      <c r="K99" s="2" t="n">
+      <c r="K99" s="3" t="n">
         <v>2.75</v>
       </c>
       <c r="L99" t="n">
@@ -5844,7 +5863,7 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="1" t="n">
+      <c r="A100" s="2" t="n">
         <v>45016</v>
       </c>
       <c r="B100" t="n">
@@ -5874,7 +5893,7 @@
       <c r="J100" t="n">
         <v>3.9</v>
       </c>
-      <c r="K100" s="2" t="n">
+      <c r="K100" s="3" t="n">
         <v>2.75</v>
       </c>
       <c r="L100" t="n">
@@ -5900,7 +5919,7 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="1" t="n">
+      <c r="A101" s="2" t="n">
         <v>45046</v>
       </c>
       <c r="B101" t="n">
@@ -5930,7 +5949,7 @@
       <c r="J101" t="n">
         <v>3.8</v>
       </c>
-      <c r="K101" s="2" t="n">
+      <c r="K101" s="3" t="n">
         <v>2.75</v>
       </c>
       <c r="L101" t="n">
@@ -5956,7 +5975,7 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="1" t="n">
+      <c r="A102" s="2" t="n">
         <v>45077</v>
       </c>
       <c r="B102" t="n">
@@ -5986,7 +6005,7 @@
       <c r="J102" t="n">
         <v>3.6</v>
       </c>
-      <c r="K102" s="2" t="n">
+      <c r="K102" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L102" t="n">
@@ -6012,7 +6031,7 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="1" t="n">
+      <c r="A103" s="2" t="n">
         <v>45107</v>
       </c>
       <c r="B103" t="n">
@@ -6042,7 +6061,7 @@
       <c r="J103" t="n">
         <v>3.5</v>
       </c>
-      <c r="K103" s="2" t="n">
+      <c r="K103" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L103" t="n">
@@ -6068,7 +6087,7 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="1" t="n">
+      <c r="A104" s="2" t="n">
         <v>45138</v>
       </c>
       <c r="B104" t="n">
@@ -6098,7 +6117,7 @@
       <c r="J104" t="n">
         <v>3.1</v>
       </c>
-      <c r="K104" s="2" t="n">
+      <c r="K104" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L104" t="n">
@@ -6124,7 +6143,7 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="1" t="n">
+      <c r="A105" s="2" t="n">
         <v>45169</v>
       </c>
       <c r="B105" t="n">
@@ -6148,39 +6167,39 @@
       <c r="H105" t="n">
         <v>85.86000061035156</v>
       </c>
-      <c r="I105" s="2" t="n">
+      <c r="I105" s="3" t="n">
         <v>1451.93994140625</v>
       </c>
       <c r="J105" t="n">
         <v>2.8</v>
       </c>
-      <c r="K105" s="2" t="n">
+      <c r="K105" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="L105" s="2" t="n">
+      <c r="L105" s="3" t="n">
         <v>3.84</v>
       </c>
-      <c r="M105" s="2" t="n">
+      <c r="M105" s="3" t="n">
         <v>163.9460213519798</v>
       </c>
-      <c r="N105" s="2" t="n">
+      <c r="N105" s="3" t="n">
         <v>110.6407541748721</v>
       </c>
-      <c r="O105" s="2" t="n">
+      <c r="O105" s="3" t="n">
         <v>166.6150576463907</v>
       </c>
-      <c r="P105" s="2" t="n">
+      <c r="P105" s="3" t="n">
         <v>2166.050340130452</v>
       </c>
-      <c r="Q105" s="2" t="n">
+      <c r="Q105" s="3" t="n">
         <v>169.9825811951376</v>
       </c>
-      <c r="R105" s="2" t="n">
+      <c r="R105" s="3" t="n">
         <v>779.5725012698099</v>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="1" t="n">
+      <c r="A106" s="2" t="n">
         <v>45199</v>
       </c>
       <c r="B106" t="n">
@@ -6210,7 +6229,7 @@
       <c r="J106" t="n">
         <v>2.5</v>
       </c>
-      <c r="K106" s="2" t="n">
+      <c r="K106" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L106" t="n">
@@ -6236,7 +6255,7 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="1" t="n">
+      <c r="A107" s="2" t="n">
         <v>45230</v>
       </c>
       <c r="B107" t="n">
@@ -6266,7 +6285,7 @@
       <c r="J107" t="n">
         <v>2.5</v>
       </c>
-      <c r="K107" s="2" t="n">
+      <c r="K107" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L107" t="n">
@@ -6292,7 +6311,7 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="1" t="n">
+      <c r="A108" s="2" t="n">
         <v>45260</v>
       </c>
       <c r="B108" t="n">
@@ -6322,7 +6341,7 @@
       <c r="J108" t="n">
         <v>2.4</v>
       </c>
-      <c r="K108" s="2" t="n">
+      <c r="K108" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L108" t="n">
@@ -6348,7 +6367,7 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="1" t="n">
+      <c r="A109" s="2" t="n">
         <v>45291</v>
       </c>
       <c r="B109" t="n">
@@ -6378,7 +6397,7 @@
       <c r="J109" t="n">
         <v>2</v>
       </c>
-      <c r="K109" s="2" t="n">
+      <c r="K109" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L109" t="n">
@@ -6404,7 +6423,7 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="1" t="n">
+      <c r="A110" s="2" t="n">
         <v>45322</v>
       </c>
       <c r="B110" t="n">
@@ -6434,7 +6453,7 @@
       <c r="J110" t="n">
         <v>1.9</v>
       </c>
-      <c r="K110" s="2" t="n">
+      <c r="K110" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L110" t="n">
@@ -6460,7 +6479,7 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="1" t="n">
+      <c r="A111" s="2" t="n">
         <v>45351</v>
       </c>
       <c r="B111" t="n">
@@ -6490,7 +6509,7 @@
       <c r="J111" t="n">
         <v>1.8</v>
       </c>
-      <c r="K111" s="2" t="n">
+      <c r="K111" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L111" t="n">
@@ -6516,7 +6535,7 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="1" t="n">
+      <c r="A112" s="2" t="n">
         <v>45382</v>
       </c>
       <c r="B112" t="n">
@@ -6525,19 +6544,19 @@
       <c r="C112" t="n">
         <v>5.375</v>
       </c>
-      <c r="D112" s="2" t="n">
+      <c r="D112" s="3" t="n">
         <v>4.205999851226807</v>
       </c>
-      <c r="E112" s="2" t="n">
+      <c r="E112" s="3" t="n">
         <v>13.01000022888184</v>
       </c>
       <c r="F112" t="n">
         <v>4.730500221252441</v>
       </c>
-      <c r="G112" s="2" t="n">
+      <c r="G112" s="3" t="n">
         <v>104.5500030517578</v>
       </c>
-      <c r="H112" s="2" t="n">
+      <c r="H112" s="3" t="n">
         <v>87.48000335693359</v>
       </c>
       <c r="I112" t="n">
@@ -6546,7 +6565,7 @@
       <c r="J112" t="n">
         <v>1.8</v>
       </c>
-      <c r="K112" s="2" t="n">
+      <c r="K112" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L112" t="n">
@@ -6572,7 +6591,7 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="1" t="n">
+      <c r="A113" s="2" t="n">
         <v>45412</v>
       </c>
       <c r="B113" t="n">
@@ -6602,7 +6621,7 @@
       <c r="J113" t="n">
         <v>1.7</v>
       </c>
-      <c r="K113" s="2" t="n">
+      <c r="K113" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L113" t="n">
@@ -6628,7 +6647,7 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="1" t="n">
+      <c r="A114" s="2" t="n">
         <v>45443</v>
       </c>
       <c r="B114" t="n">
@@ -6658,7 +6677,7 @@
       <c r="J114" t="n">
         <v>1.9</v>
       </c>
-      <c r="K114" s="2" t="n">
+      <c r="K114" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L114" t="n">
@@ -6684,7 +6703,7 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="1" t="n">
+      <c r="A115" s="2" t="n">
         <v>45473</v>
       </c>
       <c r="B115" t="n">
@@ -6714,7 +6733,7 @@
       <c r="J115" t="n">
         <v>1.9</v>
       </c>
-      <c r="K115" s="2" t="n">
+      <c r="K115" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L115" t="n">
@@ -6740,7 +6759,7 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="1" t="n">
+      <c r="A116" s="2" t="n">
         <v>45504</v>
       </c>
       <c r="B116" t="n">
@@ -6770,7 +6789,7 @@
       <c r="J116" t="n">
         <v>1.9</v>
       </c>
-      <c r="K116" s="2" t="n">
+      <c r="K116" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L116" t="n">
@@ -6796,7 +6815,7 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="1" t="n">
+      <c r="A117" s="2" t="n">
         <v>45535</v>
       </c>
       <c r="B117" t="n">
@@ -6826,7 +6845,7 @@
       <c r="J117" t="n">
         <v>1.9</v>
       </c>
-      <c r="K117" s="2" t="n">
+      <c r="K117" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L117" t="n">
@@ -6852,7 +6871,7 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="1" t="n">
+      <c r="A118" s="2" t="n">
         <v>45565</v>
       </c>
       <c r="B118" t="n">
@@ -6882,7 +6901,7 @@
       <c r="J118" t="n">
         <v>1.9</v>
       </c>
-      <c r="K118" s="2" t="n">
+      <c r="K118" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L118" t="n">
@@ -6908,7 +6927,7 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="1" t="n">
+      <c r="A119" s="2" t="n">
         <v>45596</v>
       </c>
       <c r="B119" t="n">
@@ -6932,39 +6951,39 @@
       <c r="H119" t="n">
         <v>72.55000305175781</v>
       </c>
-      <c r="I119" s="2" t="n">
+      <c r="I119" s="3" t="n">
         <v>1601.880004882812</v>
       </c>
       <c r="J119" t="n">
         <v>1.8</v>
       </c>
-      <c r="K119" s="2" t="n">
+      <c r="K119" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="L119" s="2" t="n">
+      <c r="L119" s="3" t="n">
         <v>3.92</v>
       </c>
-      <c r="M119" s="2" t="n">
+      <c r="M119" s="3" t="n">
         <v>214.6197543640977</v>
       </c>
-      <c r="N119" s="2" t="n">
+      <c r="N119" s="3" t="n">
         <v>114.9497478198026</v>
       </c>
-      <c r="O119" s="2" t="n">
+      <c r="O119" s="3" t="n">
         <v>217.8415307291696</v>
       </c>
-      <c r="P119" s="2" t="n">
+      <c r="P119" s="3" t="n">
         <v>1787.641959361786</v>
       </c>
-      <c r="Q119" s="2" t="n">
+      <c r="Q119" s="3" t="n">
         <v>153.5998670377484</v>
       </c>
-      <c r="R119" s="2" t="n">
+      <c r="R119" s="3" t="n">
         <v>959.4028545253725</v>
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="1" t="n">
+      <c r="A120" s="2" t="n">
         <v>45626</v>
       </c>
       <c r="B120" t="n">
@@ -6994,7 +7013,7 @@
       <c r="J120" t="n">
         <v>1.8</v>
       </c>
-      <c r="K120" s="2" t="n">
+      <c r="K120" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L120" t="n">
@@ -7020,7 +7039,7 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="1" t="n">
+      <c r="A121" s="2" t="n">
         <v>45657</v>
       </c>
       <c r="B121" t="n">
@@ -7050,7 +7069,7 @@
       <c r="J121" t="n">
         <v>1.8</v>
       </c>
-      <c r="K121" s="2" t="n">
+      <c r="K121" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L121" t="n">
@@ -7076,7 +7095,7 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="1" t="n">
+      <c r="A122" s="2" t="n">
         <v>45688</v>
       </c>
       <c r="B122" t="n">
@@ -7106,7 +7125,7 @@
       <c r="J122" t="n">
         <v>1.6</v>
       </c>
-      <c r="K122" s="2" t="n">
+      <c r="K122" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L122" t="n">
@@ -7132,7 +7151,7 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="1" t="n">
+      <c r="A123" s="2" t="n">
         <v>45716</v>
       </c>
       <c r="B123" t="n">
@@ -7162,7 +7181,7 @@
       <c r="J123" t="n">
         <v>1.8</v>
       </c>
-      <c r="K123" s="2" t="n">
+      <c r="K123" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L123" t="n">
@@ -7188,7 +7207,7 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="1" t="n">
+      <c r="A124" s="2" t="n">
         <v>45747</v>
       </c>
       <c r="B124" t="n">
@@ -7212,39 +7231,39 @@
       <c r="H124" t="n">
         <v>73.62999725341797</v>
       </c>
-      <c r="I124" s="2" t="n">
+      <c r="I124" s="3" t="n">
         <v>1513.650024414062</v>
       </c>
       <c r="J124" t="n">
         <v>1.9</v>
       </c>
-      <c r="K124" s="2" t="n">
+      <c r="K124" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="L124" s="2" t="n">
+      <c r="L124" s="3" t="n">
         <v>3.77</v>
       </c>
-      <c r="M124" s="2" t="n">
+      <c r="M124" s="3" t="n">
         <v>209.1178107862522</v>
       </c>
-      <c r="N124" s="2" t="n">
+      <c r="N124" s="3" t="n">
         <v>116.7757700786058</v>
       </c>
-      <c r="O124" s="2" t="n">
+      <c r="O124" s="3" t="n">
         <v>236.0877792961903</v>
       </c>
-      <c r="P124" s="2" t="n">
+      <c r="P124" s="3" t="n">
         <v>1570.898336797052</v>
       </c>
-      <c r="Q124" s="2" t="n">
+      <c r="Q124" s="3" t="n">
         <v>139.0093987390431</v>
       </c>
-      <c r="R124" s="2" t="n">
+      <c r="R124" s="3" t="n">
         <v>874.2065864780645</v>
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="1" t="n">
+      <c r="A125" s="2" t="n">
         <v>45777</v>
       </c>
       <c r="B125" t="n">
@@ -7274,7 +7293,7 @@
       <c r="J125" t="n">
         <v>1.9</v>
       </c>
-      <c r="K125" s="2" t="n">
+      <c r="K125" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L125" t="n">
@@ -7300,7 +7319,7 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="1" t="n">
+      <c r="A126" s="2" t="n">
         <v>45808</v>
       </c>
       <c r="B126" t="n">
@@ -7330,7 +7349,7 @@
       <c r="J126" t="n">
         <v>2</v>
       </c>
-      <c r="K126" s="2" t="n">
+      <c r="K126" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L126" t="n">
@@ -7356,7 +7375,7 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="1" t="n">
+      <c r="A127" s="2" t="n">
         <v>45838</v>
       </c>
       <c r="B127" t="n">
@@ -7386,7 +7405,7 @@
       <c r="J127" t="n">
         <v>1.8</v>
       </c>
-      <c r="K127" s="2" t="n">
+      <c r="K127" s="3" t="n">
         <v>3</v>
       </c>
       <c r="L127" t="n">
@@ -7412,7 +7431,7 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="1" t="n">
+      <c r="A128" s="2" t="n">
         <v>45869</v>
       </c>
       <c r="B128" t="n">
@@ -7442,7 +7461,7 @@
       <c r="J128" t="n">
         <v>1.8</v>
       </c>
-      <c r="K128" s="2" t="n">
+      <c r="K128" s="3" t="n">
         <v>2.75</v>
       </c>
       <c r="L128" t="n">
@@ -7468,7 +7487,7 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="1" t="n">
+      <c r="A129" s="2" t="n">
         <v>45900</v>
       </c>
       <c r="B129" t="n">
@@ -7498,7 +7517,7 @@
       <c r="J129" t="n">
         <v>1.8</v>
       </c>
-      <c r="K129" s="2" t="n">
+      <c r="K129" s="3" t="n">
         <v>2.75</v>
       </c>
       <c r="L129" t="n">
@@ -7524,7 +7543,7 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="1" t="n">
+      <c r="A130" s="2" t="n">
         <v>45930</v>
       </c>
       <c r="B130" t="n">
@@ -7554,7 +7573,7 @@
       <c r="J130" t="n">
         <v>2</v>
       </c>
-      <c r="K130" s="2" t="n">
+      <c r="K130" s="3" t="n">
         <v>2.75</v>
       </c>
       <c r="L130" t="n">
@@ -7580,7 +7599,7 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="1" t="n">
+      <c r="A131" s="2" t="n">
         <v>45961</v>
       </c>
       <c r="B131" t="n">
@@ -7610,7 +7629,7 @@
       <c r="J131" t="n">
         <v>2.1</v>
       </c>
-      <c r="K131" s="2" t="n">
+      <c r="K131" s="3" t="n">
         <v>2.75</v>
       </c>
       <c r="L131" t="n">
@@ -7636,7 +7655,7 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="1" t="n">
+      <c r="A132" s="2" t="n">
         <v>45991</v>
       </c>
       <c r="B132" t="n">
@@ -7666,7 +7685,7 @@
       <c r="J132" t="n">
         <v>2.2</v>
       </c>
-      <c r="K132" s="2" t="n">
+      <c r="K132" s="3" t="n">
         <v>2.75</v>
       </c>
       <c r="L132" t="n">
@@ -7692,7 +7711,7 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="1" t="n">
+      <c r="A133" s="2" t="n">
         <v>46022</v>
       </c>
       <c r="B133" t="n">
@@ -7722,7 +7741,7 @@
       <c r="J133" t="n">
         <v>2.2</v>
       </c>
-      <c r="K133" s="2" t="n">
+      <c r="K133" s="3" t="n">
         <v>2.75</v>
       </c>
       <c r="L133" t="n">
@@ -7748,7 +7767,7 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="1" t="n">
+      <c r="A134" s="2" t="n">
         <v>46053</v>
       </c>
       <c r="B134" t="n">
@@ -7778,7 +7797,7 @@
       <c r="J134" t="n">
         <v>2.3</v>
       </c>
-      <c r="K134" s="2" t="n">
+      <c r="K134" s="3" t="n">
         <v>2.75</v>
       </c>
       <c r="L134" t="n">
@@ -7804,7 +7823,7 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="1" t="n">
+      <c r="A135" s="2" t="n">
         <v>46081</v>
       </c>
       <c r="B135" t="n">
@@ -7834,7 +7853,7 @@
       <c r="J135" t="n">
         <v>2.3</v>
       </c>
-      <c r="K135" s="2" t="n">
+      <c r="K135" s="3" t="n">
         <v>2.75</v>
       </c>
       <c r="L135" t="n">
@@ -7860,7 +7879,7 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="1" t="n">
+      <c r="A136" s="2" t="n">
         <v>46112</v>
       </c>
       <c r="B136" t="n">
@@ -7890,7 +7909,7 @@
       <c r="J136" t="n">
         <v>2</v>
       </c>
-      <c r="K136" s="2" t="n">
+      <c r="K136" s="3" t="n">
         <v>2.75</v>
       </c>
       <c r="L136" t="n">
@@ -7916,7 +7935,7 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="1" t="n">
+      <c r="A137" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="B137" t="n">
@@ -7946,7 +7965,7 @@
       <c r="J137" t="n">
         <v>2.1</v>
       </c>
-      <c r="K137" s="2" t="n">
+      <c r="K137" s="3" t="n">
         <v>2.75</v>
       </c>
       <c r="L137" t="n">
@@ -7972,7 +7991,7 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="1" t="n">
+      <c r="A138" s="2" t="n">
         <v>46173</v>
       </c>
       <c r="B138" t="n">
@@ -8002,7 +8021,7 @@
       <c r="J138" t="n">
         <v>2</v>
       </c>
-      <c r="K138" s="2" t="n">
+      <c r="K138" s="3" t="n">
         <v>2.75</v>
       </c>
       <c r="L138" t="n">
@@ -8028,7 +8047,7 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="1" t="n">
+      <c r="A139" s="2" t="n">
         <v>46203</v>
       </c>
       <c r="B139" t="n">
@@ -8058,7 +8077,7 @@
       <c r="J139" t="n">
         <v>2</v>
       </c>
-      <c r="K139" s="2" t="n">
+      <c r="K139" s="3" t="n">
         <v>2.75</v>
       </c>
       <c r="L139" t="n">
@@ -8084,7 +8103,7 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="1" t="n">
+      <c r="A140" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="B140" t="n">
@@ -8114,7 +8133,7 @@
       <c r="J140" t="n">
         <v>1.9</v>
       </c>
-      <c r="K140" s="2" t="n">
+      <c r="K140" s="3" t="n">
         <v>2.75</v>
       </c>
       <c r="L140" t="n">
@@ -8140,10 +8159,10 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="1" t="n">
+      <c r="A141" s="2" t="n">
         <v>46265</v>
       </c>
-      <c r="B141" s="2" t="n">
+      <c r="B141" s="3" t="n">
         <v>1108.681095730554</v>
       </c>
       <c r="C141" t="n">
@@ -8167,10 +8186,10 @@
       <c r="I141" t="n">
         <v>1736.329956054688</v>
       </c>
-      <c r="J141" s="2" t="n">
+      <c r="J141" s="3" t="n">
         <v>1.9</v>
       </c>
-      <c r="K141" s="2" t="n">
+      <c r="K141" s="3" t="n">
         <v>2.75</v>
       </c>
       <c r="L141" t="n">

</xml_diff>

<commit_message>
charting & syntax cleanup
</commit_message>
<xml_diff>
--- a/output/MONTHLY_MASTER.xlsx
+++ b/output/MONTHLY_MASTER.xlsx
@@ -521,7 +521,7 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>reits</t>
+          <t>REITs</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
@@ -576,20 +576,20 @@
         <v>3.8</v>
       </c>
       <c r="M2" t="n">
-        <v>98.37437602833074</v>
+        <v>98.37435241312053</v>
       </c>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="n">
-        <v>102.9251421465344</v>
+        <v>102.9251333120346</v>
       </c>
       <c r="P2" t="n">
-        <v>119.1508195970458</v>
+        <v>119.1508655070364</v>
       </c>
       <c r="Q2" t="n">
-        <v>99.65451570275486</v>
+        <v>99.65450957691874</v>
       </c>
       <c r="R2" t="n">
-        <v>107.2503680961466</v>
+        <v>107.2503476708191</v>
       </c>
     </row>
     <row r="3">
@@ -628,20 +628,20 @@
         <v>3.87</v>
       </c>
       <c r="M3" t="n">
-        <v>103.7854273874596</v>
+        <v>103.7854324264138</v>
       </c>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="n">
-        <v>105.9545394870539</v>
+        <v>105.9545259663922</v>
       </c>
       <c r="P3" t="n">
-        <v>136.3440206329322</v>
+        <v>136.3440409828611</v>
       </c>
       <c r="Q3" t="n">
-        <v>107.1575206300284</v>
+        <v>107.1575164598785</v>
       </c>
       <c r="R3" t="n">
-        <v>114.8381622839634</v>
+        <v>114.8381568713302</v>
       </c>
     </row>
     <row r="4">
@@ -680,20 +680,20 @@
         <v>3.9</v>
       </c>
       <c r="M4" t="n">
-        <v>107.2269070632878</v>
+        <v>107.2268981995812</v>
       </c>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="n">
-        <v>104.5119926449099</v>
+        <v>104.51198238802</v>
       </c>
       <c r="P4" t="n">
-        <v>138.484658630668</v>
+        <v>138.4846910741614</v>
       </c>
       <c r="Q4" t="n">
-        <v>110.2192941712699</v>
+        <v>110.2193209114166</v>
       </c>
       <c r="R4" t="n">
-        <v>125.4287721041741</v>
+        <v>125.4287381519302</v>
       </c>
     </row>
     <row r="5">
@@ -732,20 +732,20 @@
         <v>3.85</v>
       </c>
       <c r="M5" t="n">
-        <v>107.2986680190774</v>
+        <v>107.2986685583297</v>
       </c>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="n">
-        <v>109.0602335550283</v>
+        <v>109.060228241279</v>
       </c>
       <c r="P5" t="n">
-        <v>161.8369111361148</v>
+        <v>161.8369482853855</v>
       </c>
       <c r="Q5" t="n">
-        <v>113.8251529477031</v>
+        <v>113.8251468684475</v>
       </c>
       <c r="R5" t="n">
-        <v>117.5916698979478</v>
+        <v>117.5917170424015</v>
       </c>
     </row>
     <row r="6">
@@ -784,20 +784,20 @@
         <v>3.91</v>
       </c>
       <c r="M6" t="n">
-        <v>103.4372726715695</v>
+        <v>103.4372897718519</v>
       </c>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="n">
-        <v>107.1257414896692</v>
+        <v>107.1257172336449</v>
       </c>
       <c r="P6" t="n">
-        <v>162.8126391432206</v>
+        <v>162.8126727881289</v>
       </c>
       <c r="Q6" t="n">
-        <v>112.8121545296498</v>
+        <v>112.8121562901202</v>
       </c>
       <c r="R6" t="n">
-        <v>111.7934065152348</v>
+        <v>111.7934227359978</v>
       </c>
     </row>
     <row r="7">
@@ -836,20 +836,20 @@
         <v>4.01</v>
       </c>
       <c r="M7" t="n">
-        <v>103.0905255704807</v>
+        <v>103.090531340004</v>
       </c>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="n">
-        <v>104.4556833232777</v>
+        <v>104.4556673562581</v>
       </c>
       <c r="P7" t="n">
-        <v>158.8971809468559</v>
+        <v>158.8971828779311</v>
       </c>
       <c r="Q7" t="n">
-        <v>113.3859502923196</v>
+        <v>113.3859446803167</v>
       </c>
       <c r="R7" t="n">
-        <v>124.5922402555099</v>
+        <v>124.5922702309507</v>
       </c>
     </row>
     <row r="8">
@@ -888,20 +888,20 @@
         <v>4.06</v>
       </c>
       <c r="M8" t="n">
-        <v>103.3021901202029</v>
+        <v>103.302176021462</v>
       </c>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="n">
-        <v>106.1342542045249</v>
+        <v>106.1342529599382</v>
       </c>
       <c r="P8" t="n">
-        <v>165.1331623534221</v>
+        <v>165.1331929909585</v>
       </c>
       <c r="Q8" t="n">
-        <v>116.3730955933355</v>
+        <v>116.3730983436907</v>
       </c>
       <c r="R8" t="n">
-        <v>130.0499014423976</v>
+        <v>130.0499230408035</v>
       </c>
     </row>
     <row r="9">
@@ -940,20 +940,20 @@
         <v>4.39</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>97.9143571997994</v>
+        <v>97.91436790685036</v>
       </c>
       <c r="N9" t="inlineStr"/>
       <c r="O9" s="3" t="n">
-        <v>103.7374199862816</v>
+        <v>103.7373899586908</v>
       </c>
       <c r="P9" s="3" t="n">
-        <v>126.3458441526099</v>
+        <v>126.3458683842429</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>114.2937159915654</v>
+        <v>114.2937057901785</v>
       </c>
       <c r="R9" s="3" t="n">
-        <v>110.8244326141899</v>
+        <v>110.8244327959167</v>
       </c>
     </row>
     <row r="10">
@@ -992,20 +992,20 @@
         <v>4.14</v>
       </c>
       <c r="M10" t="n">
-        <v>92.9977109449209</v>
+        <v>92.99771169562935</v>
       </c>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="n">
-        <v>104.3623199503137</v>
+        <v>104.3622873883022</v>
       </c>
       <c r="P10" t="n">
-        <v>132.0098103064618</v>
+        <v>132.009839613264</v>
       </c>
       <c r="Q10" t="n">
-        <v>117.0920524450819</v>
+        <v>117.0920419668925</v>
       </c>
       <c r="R10" t="n">
-        <v>124.9086093156204</v>
+        <v>124.9086172806174</v>
       </c>
     </row>
     <row r="11">
@@ -1044,20 +1044,20 @@
         <v>4.37</v>
       </c>
       <c r="M11" t="n">
-        <v>94.85493686342649</v>
+        <v>94.8549486543678</v>
       </c>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="n">
-        <v>105.9863883458672</v>
+        <v>105.9863722317266</v>
       </c>
       <c r="P11" t="n">
-        <v>156.4566252440995</v>
+        <v>156.4566706218505</v>
       </c>
       <c r="Q11" t="n">
-        <v>121.518060526265</v>
+        <v>121.5180672495698</v>
       </c>
       <c r="R11" t="n">
-        <v>144.3417349278378</v>
+        <v>144.3417347405544</v>
       </c>
     </row>
     <row r="12">
@@ -1096,20 +1096,20 @@
         <v>4.2</v>
       </c>
       <c r="M12" t="n">
-        <v>94.86997324965424</v>
+        <v>94.86997350499934</v>
       </c>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="n">
-        <v>104.3279062692368</v>
+        <v>104.3279079420143</v>
       </c>
       <c r="P12" t="n">
-        <v>167.382140770631</v>
+        <v>167.3821823018771</v>
       </c>
       <c r="Q12" t="n">
-        <v>128.9172367745547</v>
+        <v>128.9172226968794</v>
       </c>
       <c r="R12" t="n">
-        <v>138.5044308443105</v>
+        <v>138.5044373696624</v>
       </c>
     </row>
     <row r="13">
@@ -1148,20 +1148,20 @@
         <v>4.19</v>
       </c>
       <c r="M13" t="n">
-        <v>95.71995996230343</v>
+        <v>95.71995150182654</v>
       </c>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="n">
-        <v>104.8390167420868</v>
+        <v>104.8390101873304</v>
       </c>
       <c r="P13" t="n">
-        <v>169.5993805607475</v>
+        <v>169.5993971284184</v>
       </c>
       <c r="Q13" t="n">
-        <v>131.6284398111237</v>
+        <v>131.6284315770084</v>
       </c>
       <c r="R13" t="n">
-        <v>165.2180487545205</v>
+        <v>165.2180509659574</v>
       </c>
     </row>
     <row r="14">
@@ -1200,20 +1200,20 @@
         <v>3.85</v>
       </c>
       <c r="M14" t="n">
-        <v>93.39149291782198</v>
+        <v>93.39149222643324</v>
       </c>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="n">
-        <v>107.425246405806</v>
+        <v>107.4252560185794</v>
       </c>
       <c r="P14" t="n">
-        <v>157.8503216939551</v>
+        <v>157.850361035621</v>
       </c>
       <c r="Q14" t="n">
-        <v>132.850618608024</v>
+        <v>132.8506140840422</v>
       </c>
       <c r="R14" t="n">
-        <v>140.2862052164549</v>
+        <v>140.2861991479637</v>
       </c>
     </row>
     <row r="15">
@@ -1252,20 +1252,20 @@
         <v>3.92</v>
       </c>
       <c r="M15" t="n">
-        <v>96.6151449916637</v>
+        <v>96.61515540722515</v>
       </c>
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="n">
-        <v>112.998365004195</v>
+        <v>112.9983532657839</v>
       </c>
       <c r="P15" t="n">
-        <v>156.9901359466429</v>
+        <v>156.9901673184638</v>
       </c>
       <c r="Q15" t="n">
-        <v>127.1420399326788</v>
+        <v>127.1420315915643</v>
       </c>
       <c r="R15" t="n">
-        <v>153.169505750378</v>
+        <v>153.1695141132298</v>
       </c>
     </row>
     <row r="16">
@@ -1304,20 +1304,20 @@
         <v>3.78</v>
       </c>
       <c r="M16" t="n">
-        <v>102.2242692199826</v>
+        <v>102.2242743408087</v>
       </c>
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="n">
-        <v>114.4279559077895</v>
+        <v>114.4279308201674</v>
       </c>
       <c r="P16" t="n">
-        <v>161.9968620863982</v>
+        <v>161.9969147950128</v>
       </c>
       <c r="Q16" t="n">
-        <v>127.09989240178</v>
+        <v>127.0998681507231</v>
       </c>
       <c r="R16" t="n">
-        <v>163.3114869481402</v>
+        <v>163.311454393376</v>
       </c>
     </row>
     <row r="17">
@@ -1356,20 +1356,20 @@
         <v>3.88</v>
       </c>
       <c r="M17" t="n">
-        <v>100.5136961923656</v>
+        <v>100.5136855613799</v>
       </c>
       <c r="N17" t="inlineStr"/>
       <c r="O17" t="n">
-        <v>114.7335049175501</v>
+        <v>114.7334971738379</v>
       </c>
       <c r="P17" t="n">
-        <v>151.220765902201</v>
+        <v>151.2208082314584</v>
       </c>
       <c r="Q17" t="n">
-        <v>126.6434897586207</v>
+        <v>126.6434746625855</v>
       </c>
       <c r="R17" t="n">
-        <v>170.9932975602466</v>
+        <v>170.9932868619028</v>
       </c>
     </row>
     <row r="18">
@@ -1408,20 +1408,20 @@
         <v>3.92</v>
       </c>
       <c r="M18" t="n">
-        <v>97.44517528173083</v>
+        <v>97.44518759706334</v>
       </c>
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="n">
-        <v>118.644890608089</v>
+        <v>118.6449004588067</v>
       </c>
       <c r="P18" t="n">
-        <v>154.6323504141578</v>
+        <v>154.6324050847008</v>
       </c>
       <c r="Q18" t="n">
-        <v>125.0320471622586</v>
+        <v>125.0320521036864</v>
       </c>
       <c r="R18" t="n">
-        <v>175.09485044563</v>
+        <v>175.0948719598003</v>
       </c>
     </row>
     <row r="19">
@@ -1460,20 +1460,20 @@
         <v>3.75</v>
       </c>
       <c r="M19" t="n">
-        <v>97.66722106219129</v>
+        <v>97.66721710798907</v>
       </c>
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="n">
-        <v>120.4485911609294</v>
+        <v>120.4485781255417</v>
       </c>
       <c r="P19" t="n">
-        <v>149.5178139306495</v>
+        <v>149.5178493730118</v>
       </c>
       <c r="Q19" t="n">
-        <v>125.8710797071328</v>
+        <v>125.8710784560445</v>
       </c>
       <c r="R19" t="n">
-        <v>187.2039588605737</v>
+        <v>187.2039845143634</v>
       </c>
     </row>
     <row r="20">
@@ -1512,20 +1512,20 @@
         <v>3.6</v>
       </c>
       <c r="M20" t="n">
-        <v>97.48020072761986</v>
+        <v>97.4801909159526</v>
       </c>
       <c r="N20" t="inlineStr"/>
       <c r="O20" t="n">
-        <v>121.6364034208485</v>
+        <v>121.6363885335569</v>
       </c>
       <c r="P20" t="n">
-        <v>160.3381712935895</v>
+        <v>160.3382065564388</v>
       </c>
       <c r="Q20" t="n">
-        <v>125.639244190935</v>
+        <v>125.6392392447484</v>
       </c>
       <c r="R20" t="n">
-        <v>192.6504834096988</v>
+        <v>192.6505024756831</v>
       </c>
     </row>
     <row r="21">
@@ -1564,20 +1564,20 @@
         <v>3.59</v>
       </c>
       <c r="M21" s="3" t="n">
-        <v>101.6910712300357</v>
+        <v>101.6910556253835</v>
       </c>
       <c r="N21" t="inlineStr"/>
       <c r="O21" s="3" t="n">
-        <v>125.5703385582802</v>
+        <v>125.5703290778238</v>
       </c>
       <c r="P21" s="3" t="n">
-        <v>160.8174323530147</v>
+        <v>160.8174633718208</v>
       </c>
       <c r="Q21" s="3" t="n">
-        <v>127.4272877300538</v>
+        <v>127.4272803482186</v>
       </c>
       <c r="R21" s="3" t="n">
-        <v>192.8311799830827</v>
+        <v>192.8311702729623</v>
       </c>
     </row>
     <row r="22">
@@ -1616,20 +1616,20 @@
         <v>3.55</v>
       </c>
       <c r="M22" t="n">
-        <v>100.8278966283867</v>
+        <v>100.8279050240244</v>
       </c>
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="n">
-        <v>125.1852218437356</v>
+        <v>125.1852186716605</v>
       </c>
       <c r="P22" t="n">
-        <v>160.9422887330792</v>
+        <v>160.9423260976588</v>
       </c>
       <c r="Q22" t="n">
-        <v>127.0650941375464</v>
+        <v>127.0650836530197</v>
       </c>
       <c r="R22" t="n">
-        <v>214.4159468133514</v>
+        <v>214.4158989623239</v>
       </c>
     </row>
     <row r="23">
@@ -1668,20 +1668,20 @@
         <v>3.61</v>
       </c>
       <c r="M23" t="n">
-        <v>104.9686640195653</v>
+        <v>104.9686530019274</v>
       </c>
       <c r="N23" t="inlineStr"/>
       <c r="O23" t="n">
-        <v>128.8551602830469</v>
+        <v>128.855121543894</v>
       </c>
       <c r="P23" t="n">
-        <v>161.2025323560031</v>
+        <v>161.2025976966638</v>
       </c>
       <c r="Q23" t="n">
-        <v>129.3323375884117</v>
+        <v>129.3323231424372</v>
       </c>
       <c r="R23" t="n">
-        <v>213.1240357409403</v>
+        <v>213.1240928880147</v>
       </c>
     </row>
     <row r="24">
@@ -1720,20 +1720,20 @@
         <v>4.35</v>
       </c>
       <c r="M24" t="n">
-        <v>100.6919044033506</v>
+        <v>100.6919032797179</v>
       </c>
       <c r="N24" t="inlineStr"/>
       <c r="O24" t="n">
-        <v>124.1260342824857</v>
+        <v>124.1260092071735</v>
       </c>
       <c r="P24" t="n">
-        <v>161.425639277013</v>
+        <v>161.425674016797</v>
       </c>
       <c r="Q24" t="n">
-        <v>126.1930297611235</v>
+        <v>126.193016567386</v>
       </c>
       <c r="R24" t="n">
-        <v>229.972952592769</v>
+        <v>229.9730049430111</v>
       </c>
     </row>
     <row r="25">
@@ -1772,20 +1772,20 @@
         <v>4.22</v>
       </c>
       <c r="M25" t="n">
-        <v>102.3427103807533</v>
+        <v>102.3427116603758</v>
       </c>
       <c r="N25" t="inlineStr"/>
       <c r="O25" t="n">
-        <v>128.1423264532299</v>
+        <v>128.142287604888</v>
       </c>
       <c r="P25" t="n">
-        <v>170.9327806992009</v>
+        <v>170.9328046579934</v>
       </c>
       <c r="Q25" t="n">
-        <v>129.257896781856</v>
+        <v>129.2578825667346</v>
       </c>
       <c r="R25" t="n">
-        <v>226.0250857129951</v>
+        <v>226.0251473102865</v>
       </c>
     </row>
     <row r="26">
@@ -1824,20 +1824,20 @@
         <v>4.14</v>
       </c>
       <c r="M26" t="n">
-        <v>106.5026995855452</v>
+        <v>106.5026944496907</v>
       </c>
       <c r="N26" t="inlineStr"/>
       <c r="O26" t="n">
-        <v>131.7047078576626</v>
+        <v>131.7046669808429</v>
       </c>
       <c r="P26" t="n">
-        <v>180.2204389949512</v>
+        <v>180.2204923419858</v>
       </c>
       <c r="Q26" t="n">
-        <v>128.8888555768681</v>
+        <v>128.8888500812333</v>
       </c>
       <c r="R26" t="n">
-        <v>255.4750028839361</v>
+        <v>255.4749715774079</v>
       </c>
     </row>
     <row r="27">
@@ -1876,20 +1876,20 @@
         <v>4.04</v>
       </c>
       <c r="M27" t="n">
-        <v>108.4766406125146</v>
+        <v>108.4766364113775</v>
       </c>
       <c r="N27" t="inlineStr"/>
       <c r="O27" t="n">
-        <v>127.5850801392847</v>
+        <v>127.5850664677137</v>
       </c>
       <c r="P27" t="n">
-        <v>201.5675477957122</v>
+        <v>201.5676005619055</v>
       </c>
       <c r="Q27" t="n">
-        <v>129.5697622742317</v>
+        <v>129.5697670344082</v>
       </c>
       <c r="R27" t="n">
-        <v>276.8609220815716</v>
+        <v>276.8609850423358</v>
       </c>
     </row>
     <row r="28">
@@ -1928,20 +1928,20 @@
         <v>4.13</v>
       </c>
       <c r="M28" t="n">
-        <v>114.8296276397322</v>
+        <v>114.8296224671624</v>
       </c>
       <c r="N28" t="inlineStr"/>
       <c r="O28" t="n">
-        <v>129.6918331004231</v>
+        <v>129.6918335723266</v>
       </c>
       <c r="P28" t="n">
-        <v>225.640418323653</v>
+        <v>225.6404345775087</v>
       </c>
       <c r="Q28" t="n">
-        <v>132.4758687064073</v>
+        <v>132.4758718770172</v>
       </c>
       <c r="R28" t="n">
-        <v>284.1496615730298</v>
+        <v>284.1496838719969</v>
       </c>
     </row>
     <row r="29">
@@ -1980,20 +1980,20 @@
         <v>4.05</v>
       </c>
       <c r="M29" t="n">
-        <v>118.927018257988</v>
+        <v>118.927021139412</v>
       </c>
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="n">
-        <v>128.9234059388846</v>
+        <v>128.9233721881446</v>
       </c>
       <c r="P29" t="n">
-        <v>245.5287334179388</v>
+        <v>245.5288386826826</v>
       </c>
       <c r="Q29" t="n">
-        <v>127.4250793785155</v>
+        <v>127.4250864497548</v>
       </c>
       <c r="R29" t="n">
-        <v>288.1719772432739</v>
+        <v>288.1720141601268</v>
       </c>
     </row>
     <row r="30">
@@ -2032,20 +2032,20 @@
         <v>3.87</v>
       </c>
       <c r="M30" t="n">
-        <v>123.9146788664846</v>
+        <v>123.9146663358798</v>
       </c>
       <c r="N30" t="inlineStr"/>
       <c r="O30" t="n">
-        <v>128.8062245783404</v>
+        <v>128.8062469751864</v>
       </c>
       <c r="P30" t="n">
-        <v>262.6933528747732</v>
+        <v>262.69340801526</v>
       </c>
       <c r="Q30" t="n">
-        <v>129.4759062673889</v>
+        <v>129.4759106555026</v>
       </c>
       <c r="R30" t="n">
-        <v>290.8278661748305</v>
+        <v>290.8279023292222</v>
       </c>
     </row>
     <row r="31">
@@ -2084,20 +2084,20 @@
         <v>3.91</v>
       </c>
       <c r="M31" t="n">
-        <v>126.4622187945492</v>
+        <v>126.4622093578761</v>
       </c>
       <c r="N31" t="inlineStr"/>
       <c r="O31" t="n">
-        <v>134.3880087267182</v>
+        <v>134.3879684085865</v>
       </c>
       <c r="P31" t="n">
-        <v>299.5791006663201</v>
+        <v>299.5791662589999</v>
       </c>
       <c r="Q31" t="n">
-        <v>127.2420662907164</v>
+        <v>127.2420651987168</v>
       </c>
       <c r="R31" t="n">
-        <v>310.6826310002718</v>
+        <v>310.6826702694797</v>
       </c>
     </row>
     <row r="32">
@@ -2136,20 +2136,20 @@
         <v>3.99</v>
       </c>
       <c r="M32" t="n">
-        <v>125.8290569336541</v>
+        <v>125.829028678091</v>
       </c>
       <c r="N32" t="inlineStr"/>
       <c r="O32" t="n">
-        <v>130.6500169889564</v>
+        <v>130.6499932481345</v>
       </c>
       <c r="P32" t="n">
-        <v>358.4796339235907</v>
+        <v>358.4797240419714</v>
       </c>
       <c r="Q32" t="n">
-        <v>126.2873005503289</v>
+        <v>126.2873096805411</v>
       </c>
       <c r="R32" t="n">
-        <v>321.9735340465447</v>
+        <v>321.9736316093327</v>
       </c>
     </row>
     <row r="33">
@@ -2188,20 +2188,20 @@
         <v>3.89</v>
       </c>
       <c r="M33" t="n">
-        <v>130.0740233098945</v>
+        <v>130.0740281802776</v>
       </c>
       <c r="N33" t="inlineStr"/>
       <c r="O33" t="n">
-        <v>132.3059497684263</v>
+        <v>132.3059087660324</v>
       </c>
       <c r="P33" t="n">
-        <v>351.2769895270311</v>
+        <v>351.2770725678774</v>
       </c>
       <c r="Q33" t="n">
-        <v>128.9823657070818</v>
+        <v>128.9823706860797</v>
       </c>
       <c r="R33" t="n">
-        <v>358.6836028627936</v>
+        <v>358.6836158265253</v>
       </c>
     </row>
     <row r="34">
@@ -2240,20 +2240,20 @@
         <v>3.92</v>
       </c>
       <c r="M34" t="n">
-        <v>126.1729864435245</v>
+        <v>126.1729698308357</v>
       </c>
       <c r="N34" t="inlineStr"/>
       <c r="O34" t="n">
-        <v>134.9772222283217</v>
+        <v>134.9772047105333</v>
       </c>
       <c r="P34" t="n">
-        <v>364.5699084055543</v>
+        <v>364.56999731877</v>
       </c>
       <c r="Q34" t="n">
-        <v>128.7377148577233</v>
+        <v>128.7377192008835</v>
       </c>
       <c r="R34" t="n">
-        <v>365.8627627982685</v>
+        <v>365.8627718475248</v>
       </c>
     </row>
     <row r="35">
@@ -2292,20 +2292,20 @@
         <v>3.94</v>
       </c>
       <c r="M35" t="n">
-        <v>124.759287700689</v>
+        <v>124.7592791128298</v>
       </c>
       <c r="N35" t="inlineStr"/>
       <c r="O35" t="n">
-        <v>132.4268447801565</v>
+        <v>132.4268417956351</v>
       </c>
       <c r="P35" t="n">
-        <v>407.256651225758</v>
+        <v>407.2568242476109</v>
       </c>
       <c r="Q35" t="n">
-        <v>128.9863008348534</v>
+        <v>128.9862983543279</v>
       </c>
       <c r="R35" t="n">
-        <v>426.6522238300648</v>
+        <v>426.6522381284307</v>
       </c>
     </row>
     <row r="36">
@@ -2344,22 +2344,22 @@
         <v>3.89</v>
       </c>
       <c r="M36" t="n">
-        <v>123.040618352046</v>
+        <v>123.0406191204165</v>
       </c>
       <c r="N36" t="n">
         <v>100</v>
       </c>
       <c r="O36" t="n">
-        <v>131.0029776667184</v>
+        <v>131.002967965358</v>
       </c>
       <c r="P36" t="n">
-        <v>428.7416502617614</v>
+        <v>428.741756020617</v>
       </c>
       <c r="Q36" t="n">
-        <v>125.3181878179334</v>
+        <v>125.3182064797862</v>
       </c>
       <c r="R36" t="n">
-        <v>475.2096263088946</v>
+        <v>475.2096719155409</v>
       </c>
     </row>
     <row r="37">
@@ -2398,22 +2398,22 @@
         <v>3.91</v>
       </c>
       <c r="M37" t="n">
-        <v>130.6636254036307</v>
+        <v>130.6636172683421</v>
       </c>
       <c r="N37" t="n">
-        <v>107.9068546280969</v>
+        <v>107.9068535967807</v>
       </c>
       <c r="O37" t="n">
-        <v>146.1028426782606</v>
+        <v>146.1028239065589</v>
       </c>
       <c r="P37" t="n">
-        <v>483.9687928172983</v>
+        <v>483.9690157749015</v>
       </c>
       <c r="Q37" t="n">
-        <v>131.2691762845809</v>
+        <v>131.2691748118108</v>
       </c>
       <c r="R37" t="n">
-        <v>529.0482159976658</v>
+        <v>529.0481624678202</v>
       </c>
     </row>
     <row r="38">
@@ -2452,22 +2452,22 @@
         <v>3.96</v>
       </c>
       <c r="M38" s="3" t="n">
-        <v>139.2056070289008</v>
+        <v>139.2056164180506</v>
       </c>
       <c r="N38" s="3" t="n">
-        <v>106.3690987258629</v>
+        <v>106.3691083949243</v>
       </c>
       <c r="O38" s="3" t="n">
-        <v>131.3477012859881</v>
+        <v>131.3476733803591</v>
       </c>
       <c r="P38" s="3" t="n">
-        <v>481.752107018418</v>
+        <v>481.7522264914951</v>
       </c>
       <c r="Q38" s="3" t="n">
-        <v>135.6503114629042</v>
+        <v>135.6503149036956</v>
       </c>
       <c r="R38" s="3" t="n">
-        <v>594.7357734359055</v>
+        <v>594.7357518404923</v>
       </c>
     </row>
     <row r="39">
@@ -2506,22 +2506,22 @@
         <v>4.01</v>
       </c>
       <c r="M39" t="n">
-        <v>142.6418548071572</v>
+        <v>142.6418369256956</v>
       </c>
       <c r="N39" t="n">
-        <v>105.1654960450411</v>
+        <v>105.1654984669877</v>
       </c>
       <c r="O39" t="n">
-        <v>131.4189733350582</v>
+        <v>131.4189668618227</v>
       </c>
       <c r="P39" t="n">
-        <v>495.1228197116939</v>
+        <v>495.1229502711499</v>
       </c>
       <c r="Q39" t="n">
-        <v>137.0151304593779</v>
+        <v>137.0150992049531</v>
       </c>
       <c r="R39" t="n">
-        <v>610.1139211225728</v>
+        <v>610.1138713830129</v>
       </c>
     </row>
     <row r="40">
@@ -2560,22 +2560,22 @@
         <v>3.94</v>
       </c>
       <c r="M40" t="n">
-        <v>146.9024355708899</v>
+        <v>146.9024138460866</v>
       </c>
       <c r="N40" t="n">
-        <v>109.0363194717368</v>
+        <v>109.0363073319148</v>
       </c>
       <c r="O40" t="n">
-        <v>125.9931769968926</v>
+        <v>125.9932024296885</v>
       </c>
       <c r="P40" t="n">
-        <v>422.1023783325818</v>
+        <v>422.1024574773255</v>
       </c>
       <c r="Q40" t="n">
-        <v>139.2007895427029</v>
+        <v>139.2008118955735</v>
       </c>
       <c r="R40" t="n">
-        <v>526.8910839361474</v>
+        <v>526.8910107257163</v>
       </c>
     </row>
     <row r="41">
@@ -2614,22 +2614,22 @@
         <v>4.13</v>
       </c>
       <c r="M41" t="n">
-        <v>147.4341001219557</v>
+        <v>147.4340920994775</v>
       </c>
       <c r="N41" t="n">
-        <v>109.5091700026762</v>
+        <v>109.5091684597308</v>
       </c>
       <c r="O41" t="n">
-        <v>130.984770963947</v>
+        <v>130.9847594956829</v>
       </c>
       <c r="P41" t="n">
-        <v>404.2394434326137</v>
+        <v>404.2395951143506</v>
       </c>
       <c r="Q41" t="n">
-        <v>144.1461566740602</v>
+        <v>144.1461671038865</v>
       </c>
       <c r="R41" t="n">
-        <v>556.1193746255175</v>
+        <v>556.1194588936313</v>
       </c>
     </row>
     <row r="42">
@@ -2668,22 +2668,22 @@
         <v>4.18</v>
       </c>
       <c r="M42" t="n">
-        <v>133.2035878155643</v>
+        <v>133.2035852260922</v>
       </c>
       <c r="N42" t="n">
-        <v>107.0029715175125</v>
+        <v>107.0029720569263</v>
       </c>
       <c r="O42" t="n">
-        <v>138.5566937275216</v>
+        <v>138.5566807474393</v>
       </c>
       <c r="P42" t="n">
-        <v>471.1890352954501</v>
+        <v>471.1892087500866</v>
       </c>
       <c r="Q42" t="n">
-        <v>136.4009662723353</v>
+        <v>136.4009904234624</v>
       </c>
       <c r="R42" t="n">
-        <v>548.5945234216981</v>
+        <v>548.5945171348111</v>
       </c>
     </row>
     <row r="43">
@@ -2722,22 +2722,22 @@
         <v>4.2</v>
       </c>
       <c r="M43" t="n">
-        <v>127.5630989144999</v>
+        <v>127.5631042057019</v>
       </c>
       <c r="N43" t="n">
-        <v>104.2725350907116</v>
+        <v>104.2725520275478</v>
       </c>
       <c r="O43" t="n">
-        <v>142.8332407099051</v>
+        <v>142.833225335293</v>
       </c>
       <c r="P43" t="n">
-        <v>467.6744070310234</v>
+        <v>467.6745281688914</v>
       </c>
       <c r="Q43" t="n">
-        <v>139.4605821749018</v>
+        <v>139.4605496607436</v>
       </c>
       <c r="R43" t="n">
-        <v>600.6630922662885</v>
+        <v>600.6630549006987</v>
       </c>
     </row>
     <row r="44">
@@ -2776,22 +2776,22 @@
         <v>4.07</v>
       </c>
       <c r="M44" t="n">
-        <v>135.7489297519348</v>
+        <v>135.7489377421829</v>
       </c>
       <c r="N44" t="n">
-        <v>105.4892656382484</v>
+        <v>105.4892597347121</v>
       </c>
       <c r="O44" t="n">
-        <v>140.9010306433491</v>
+        <v>140.9009984635527</v>
       </c>
       <c r="P44" t="n">
-        <v>548.3297633450367</v>
+        <v>548.3300286410381</v>
       </c>
       <c r="Q44" t="n">
-        <v>150.3657890659052</v>
+        <v>150.3657810341981</v>
       </c>
       <c r="R44" t="n">
-        <v>583.2114363143864</v>
+        <v>583.2115429774009</v>
       </c>
     </row>
     <row r="45">
@@ -2830,22 +2830,22 @@
         <v>4.04</v>
       </c>
       <c r="M45" s="3" t="n">
-        <v>140.3911315882537</v>
+        <v>140.3911295780967</v>
       </c>
       <c r="N45" s="3" t="n">
-        <v>105.374234555994</v>
+        <v>105.3742421070274</v>
       </c>
       <c r="O45" s="3" t="n">
-        <v>141.4153321382273</v>
+        <v>141.4153006213441</v>
       </c>
       <c r="P45" s="3" t="n">
-        <v>662.7670105801706</v>
+        <v>662.7671940992731</v>
       </c>
       <c r="Q45" s="3" t="n">
-        <v>154.9234626415269</v>
+        <v>154.9234408775778</v>
       </c>
       <c r="R45" s="3" t="n">
-        <v>625.4760320899331</v>
+        <v>625.4760372845677</v>
       </c>
     </row>
     <row r="46">
@@ -2884,22 +2884,22 @@
         <v>4.07</v>
       </c>
       <c r="M46" t="n">
-        <v>141.6206386162927</v>
+        <v>141.6206375231348</v>
       </c>
       <c r="N46" t="n">
-        <v>106.1477705281806</v>
+        <v>106.1477653572969</v>
       </c>
       <c r="O46" t="n">
-        <v>138.7948428606034</v>
+        <v>138.7948253799666</v>
       </c>
       <c r="P46" t="n">
-        <v>690.0453649931553</v>
+        <v>690.0455439308746</v>
       </c>
       <c r="Q46" t="n">
-        <v>153.4466249111017</v>
+        <v>153.4466175906661</v>
       </c>
       <c r="R46" t="n">
-        <v>604.7792134807028</v>
+        <v>604.7793701667654</v>
       </c>
     </row>
     <row r="47">
@@ -2938,22 +2938,22 @@
         <v>4.08</v>
       </c>
       <c r="M47" t="n">
-        <v>137.2267337282742</v>
+        <v>137.2267386859551</v>
       </c>
       <c r="N47" t="n">
-        <v>105.5678527924399</v>
+        <v>105.5678559373695</v>
       </c>
       <c r="O47" t="n">
-        <v>138.8775049794343</v>
+        <v>138.8775199276695</v>
       </c>
       <c r="P47" t="n">
-        <v>619.5022751209937</v>
+        <v>619.5024510819627</v>
       </c>
       <c r="Q47" t="n">
-        <v>151.3406245076502</v>
+        <v>151.3406207237485</v>
       </c>
       <c r="R47" t="n">
-        <v>637.8591771642966</v>
+        <v>637.8591939297022</v>
       </c>
     </row>
     <row r="48">
@@ -2992,22 +2992,22 @@
         <v>4.12</v>
       </c>
       <c r="M48" t="n">
-        <v>137.6815330531751</v>
+        <v>137.6815139436231</v>
       </c>
       <c r="N48" t="n">
-        <v>99.27226112720537</v>
+        <v>99.27227076808762</v>
       </c>
       <c r="O48" t="n">
-        <v>140.7496858659614</v>
+        <v>140.7496584916715</v>
       </c>
       <c r="P48" t="n">
-        <v>573.8437191805967</v>
+        <v>573.8438203833832</v>
       </c>
       <c r="Q48" t="n">
-        <v>152.028257204842</v>
+        <v>152.0282615147312</v>
       </c>
       <c r="R48" t="n">
-        <v>634.7136036208626</v>
+        <v>634.7137251446064</v>
       </c>
     </row>
     <row r="49">
@@ -3046,22 +3046,22 @@
         <v>4.07</v>
       </c>
       <c r="M49" t="n">
-        <v>137.5859993234469</v>
+        <v>137.5860030313972</v>
       </c>
       <c r="N49" t="n">
-        <v>102.6181163830983</v>
+        <v>102.6181026755944</v>
       </c>
       <c r="O49" t="n">
-        <v>143.5138316934419</v>
+        <v>143.5138046186817</v>
       </c>
       <c r="P49" t="n">
-        <v>518.7560189645983</v>
+        <v>518.7561987228327</v>
       </c>
       <c r="Q49" t="n">
-        <v>155.519879075689</v>
+        <v>155.5198661230878</v>
       </c>
       <c r="R49" t="n">
-        <v>621.9053131418091</v>
+        <v>621.9054997972504</v>
       </c>
     </row>
     <row r="50">
@@ -3100,22 +3100,22 @@
         <v>4.06</v>
       </c>
       <c r="M50" t="n">
-        <v>137.1141179529078</v>
+        <v>137.1141146519014</v>
       </c>
       <c r="N50" t="n">
-        <v>107.079581562829</v>
+        <v>107.0795765205354</v>
       </c>
       <c r="O50" t="n">
-        <v>146.3714057254648</v>
+        <v>146.3713786798411</v>
       </c>
       <c r="P50" t="n">
-        <v>565.6036611738638</v>
+        <v>565.6038414457677</v>
       </c>
       <c r="Q50" t="n">
-        <v>147.6605936652062</v>
+        <v>147.6605830250249</v>
       </c>
       <c r="R50" t="n">
-        <v>548.8876350888293</v>
+        <v>548.8876749810772</v>
       </c>
     </row>
     <row r="51">
@@ -3156,22 +3156,22 @@
         <v>3.89</v>
       </c>
       <c r="M51" t="n">
-        <v>139.3360295159207</v>
+        <v>139.336016098401</v>
       </c>
       <c r="N51" t="n">
-        <v>105.8990982741809</v>
+        <v>105.8990978703931</v>
       </c>
       <c r="O51" t="n">
-        <v>147.8178189175125</v>
+        <v>147.8178109967531</v>
       </c>
       <c r="P51" t="n">
-        <v>604.9360131960926</v>
+        <v>604.9361540643881</v>
       </c>
       <c r="Q51" t="n">
-        <v>152.8088880225494</v>
+        <v>152.8088849608141</v>
       </c>
       <c r="R51" t="n">
-        <v>528.6764878370431</v>
+        <v>528.6764919306338</v>
       </c>
     </row>
     <row r="52">
@@ -3212,22 +3212,22 @@
         <v>3.77</v>
       </c>
       <c r="M52" t="n">
-        <v>130.6616703721792</v>
+        <v>130.6616606042844</v>
       </c>
       <c r="N52" t="n">
-        <v>105.4786710425316</v>
+        <v>105.478670226392</v>
       </c>
       <c r="O52" t="n">
-        <v>151.5706974833536</v>
+        <v>151.5706880919802</v>
       </c>
       <c r="P52" t="n">
-        <v>626.9114835142444</v>
+        <v>626.9116916366936</v>
       </c>
       <c r="Q52" t="n">
-        <v>149.979311430675</v>
+        <v>149.9793342422717</v>
       </c>
       <c r="R52" t="n">
-        <v>552.554169596658</v>
+        <v>552.5542374534298</v>
       </c>
     </row>
     <row r="53">
@@ -3268,22 +3268,22 @@
         <v>3.79</v>
       </c>
       <c r="M53" t="n">
-        <v>130.347109655978</v>
+        <v>130.3471179273247</v>
       </c>
       <c r="N53" t="n">
-        <v>106.7890574680307</v>
+        <v>106.7890706719482</v>
       </c>
       <c r="O53" t="n">
-        <v>153.3841465628069</v>
+        <v>153.3841037737506</v>
       </c>
       <c r="P53" t="n">
-        <v>725.9722963612192</v>
+        <v>725.9724894465655</v>
       </c>
       <c r="Q53" t="n">
-        <v>147.6443771534986</v>
+        <v>147.6443520180634</v>
       </c>
       <c r="R53" t="n">
-        <v>582.3533404748941</v>
+        <v>582.3533900285554</v>
       </c>
     </row>
     <row r="54">
@@ -3324,22 +3324,22 @@
         <v>3.78</v>
       </c>
       <c r="M54" t="n">
-        <v>132.90096795989</v>
+        <v>132.9009840516329</v>
       </c>
       <c r="N54" t="n">
-        <v>101.9514993282087</v>
+        <v>101.951498264409</v>
       </c>
       <c r="O54" t="n">
-        <v>155.5749945054434</v>
+        <v>155.5749614035297</v>
       </c>
       <c r="P54" t="n">
-        <v>674.3001397141868</v>
+        <v>674.3004136992541</v>
       </c>
       <c r="Q54" t="n">
-        <v>146.9686731343774</v>
+        <v>146.9686700871717</v>
       </c>
       <c r="R54" t="n">
-        <v>576.408942641971</v>
+        <v>576.4089002384981</v>
       </c>
     </row>
     <row r="55">
@@ -3380,22 +3380,22 @@
         <v>3.63</v>
       </c>
       <c r="M55" t="n">
-        <v>132.0036624335498</v>
+        <v>132.0036676533708</v>
       </c>
       <c r="N55" t="n">
-        <v>103.1095661904614</v>
+        <v>103.109567990558</v>
       </c>
       <c r="O55" t="n">
-        <v>157.395785525107</v>
+        <v>157.3957521180607</v>
       </c>
       <c r="P55" t="n">
-        <v>700.780879920188</v>
+        <v>700.7811873826254</v>
       </c>
       <c r="Q55" t="n">
-        <v>146.7028070984747</v>
+        <v>146.7028029874216</v>
       </c>
       <c r="R55" t="n">
-        <v>564.3525495280071</v>
+        <v>564.3525845362965</v>
       </c>
     </row>
     <row r="56">
@@ -3436,22 +3436,22 @@
         <v>3.57</v>
       </c>
       <c r="M56" t="n">
-        <v>126.3232876245427</v>
+        <v>126.3233045360541</v>
       </c>
       <c r="N56" t="n">
-        <v>99.36476685094185</v>
+        <v>99.36476408527804</v>
       </c>
       <c r="O56" t="n">
-        <v>159.3203429778185</v>
+        <v>159.3202938113228</v>
       </c>
       <c r="P56" t="n">
-        <v>746.5162255098575</v>
+        <v>746.5165752644841</v>
       </c>
       <c r="Q56" t="n">
-        <v>134.22115393268</v>
+        <v>134.2211227773932</v>
       </c>
       <c r="R56" t="n">
-        <v>554.201380061883</v>
+        <v>554.2014193499281</v>
       </c>
     </row>
     <row r="57">
@@ -3492,22 +3492,22 @@
         <v>3.32</v>
       </c>
       <c r="M57" t="n">
-        <v>123.9469070524953</v>
+        <v>123.9468984536766</v>
       </c>
       <c r="N57" t="n">
-        <v>104.3048414377182</v>
+        <v>104.3048349383143</v>
       </c>
       <c r="O57" t="n">
-        <v>168.1140467658609</v>
+        <v>168.1140435107307</v>
       </c>
       <c r="P57" t="n">
-        <v>745.6462541499773</v>
+        <v>745.6465550333528</v>
       </c>
       <c r="Q57" t="n">
-        <v>130.4420536702617</v>
+        <v>130.4420373738354</v>
       </c>
       <c r="R57" t="n">
-        <v>590.0479999073136</v>
+        <v>590.0479861990748</v>
       </c>
     </row>
     <row r="58">
@@ -3548,22 +3548,22 @@
         <v>3.32</v>
       </c>
       <c r="M58" t="n">
-        <v>123.5424173905632</v>
+        <v>123.5424204929133</v>
       </c>
       <c r="N58" t="n">
-        <v>101.4397071002201</v>
+        <v>101.4397051339134</v>
       </c>
       <c r="O58" t="n">
-        <v>166.4831083053149</v>
+        <v>166.4830931447921</v>
       </c>
       <c r="P58" t="n">
-        <v>823.0181291829148</v>
+        <v>823.0183903742957</v>
       </c>
       <c r="Q58" t="n">
-        <v>137.3367200269572</v>
+        <v>137.3367221736694</v>
       </c>
       <c r="R58" t="n">
-        <v>562.5842315912732</v>
+        <v>562.584215808046</v>
       </c>
     </row>
     <row r="59">
@@ -3604,22 +3604,22 @@
         <v>3.41</v>
       </c>
       <c r="M59" t="n">
-        <v>127.4444812295567</v>
+        <v>127.4444859166779</v>
       </c>
       <c r="N59" t="n">
-        <v>100.2415218444503</v>
+        <v>100.2415046674174</v>
       </c>
       <c r="O59" t="n">
-        <v>159.2547462714998</v>
+        <v>159.2547222694569</v>
       </c>
       <c r="P59" t="n">
-        <v>885.1509153584175</v>
+        <v>885.15120713339</v>
       </c>
       <c r="Q59" t="n">
-        <v>137.6051200912013</v>
+        <v>137.6051346773174</v>
       </c>
       <c r="R59" t="n">
-        <v>556.3695079197024</v>
+        <v>556.3695463076609</v>
       </c>
     </row>
     <row r="60">
@@ -3660,22 +3660,22 @@
         <v>3.42</v>
       </c>
       <c r="M60" t="n">
-        <v>125.1405570089147</v>
+        <v>125.1405582976115</v>
       </c>
       <c r="N60" t="n">
-        <v>103.5306678161132</v>
+        <v>103.5306551242321</v>
       </c>
       <c r="O60" t="n">
-        <v>163.1831388309033</v>
+        <v>163.1831343307076</v>
       </c>
       <c r="P60" t="n">
-        <v>874.3975519050095</v>
+        <v>874.3978439009703</v>
       </c>
       <c r="Q60" t="n">
-        <v>130.8143134980911</v>
+        <v>130.8143181597481</v>
       </c>
       <c r="R60" t="n">
-        <v>562.697108680239</v>
+        <v>562.6970293463339</v>
       </c>
     </row>
     <row r="61">
@@ -3716,22 +3716,22 @@
         <v>3.3</v>
       </c>
       <c r="M61" t="n">
-        <v>125.0871025764608</v>
+        <v>125.087091146581</v>
       </c>
       <c r="N61" t="n">
-        <v>111.1020959201747</v>
+        <v>111.1020894514236</v>
       </c>
       <c r="O61" t="n">
-        <v>160.5442638794904</v>
+        <v>160.5442564974287</v>
       </c>
       <c r="P61" t="n">
-        <v>910.0522574668936</v>
+        <v>910.0527563558766</v>
       </c>
       <c r="Q61" t="n">
-        <v>137.1895831485792</v>
+        <v>137.1895770351216</v>
       </c>
       <c r="R61" t="n">
-        <v>575.6901203547181</v>
+        <v>575.6900688507883</v>
       </c>
     </row>
     <row r="62">
@@ -3772,22 +3772,22 @@
         <v>3.13</v>
       </c>
       <c r="M62" t="n">
-        <v>120.5205263710651</v>
+        <v>120.5205147296369</v>
       </c>
       <c r="N62" t="n">
-        <v>105.5018771886446</v>
+        <v>105.5018798846095</v>
       </c>
       <c r="O62" t="n">
-        <v>161.0046676603215</v>
+        <v>161.0046689266057</v>
       </c>
       <c r="P62" t="n">
-        <v>981.0308966655546</v>
+        <v>981.0313590388134</v>
       </c>
       <c r="Q62" t="n">
-        <v>126.3063536086563</v>
+        <v>126.3063635687722</v>
       </c>
       <c r="R62" t="n">
-        <v>660.2841435719021</v>
+        <v>660.2841369229099</v>
       </c>
     </row>
     <row r="63">
@@ -3828,22 +3828,22 @@
         <v>2.82</v>
       </c>
       <c r="M63" t="n">
-        <v>116.3340348798064</v>
+        <v>116.3340297358178</v>
       </c>
       <c r="N63" t="n">
-        <v>100.4157804933256</v>
+        <v>100.4157658322614</v>
       </c>
       <c r="O63" t="n">
-        <v>168.8880054907304</v>
+        <v>168.8879830510373</v>
       </c>
       <c r="P63" t="n">
-        <v>873.5945676953346</v>
+        <v>873.5949303866739</v>
       </c>
       <c r="Q63" t="n">
-        <v>123.8707496958992</v>
+        <v>123.8707485504625</v>
       </c>
       <c r="R63" t="n">
-        <v>634.4696704469986</v>
+        <v>634.469754989343</v>
       </c>
     </row>
     <row r="64">
@@ -3884,22 +3884,22 @@
         <v>3.35</v>
       </c>
       <c r="M64" t="n">
-        <v>100.9657878890971</v>
+        <v>100.9657909410796</v>
       </c>
       <c r="N64" t="n">
-        <v>98.15455148109022</v>
+        <v>98.15455245832322</v>
       </c>
       <c r="O64" t="n">
-        <v>146.6845967043971</v>
+        <v>146.6845799295042</v>
       </c>
       <c r="P64" t="n">
-        <v>753.044949819346</v>
+        <v>753.0450754717348</v>
       </c>
       <c r="Q64" t="n">
-        <v>118.1931764623415</v>
+        <v>118.1931642685405</v>
       </c>
       <c r="R64" t="n">
-        <v>575.0329452722796</v>
+        <v>575.0329499182005</v>
       </c>
     </row>
     <row r="65">
@@ -3940,22 +3940,22 @@
         <v>2.89</v>
       </c>
       <c r="M65" t="n">
-        <v>102.878046874819</v>
+        <v>102.8780332334752</v>
       </c>
       <c r="N65" t="n">
-        <v>99.2186992246417</v>
+        <v>99.21869505775395</v>
       </c>
       <c r="O65" t="n">
-        <v>150.693833533551</v>
+        <v>150.6938083422704</v>
       </c>
       <c r="P65" t="n">
-        <v>891.8020513876709</v>
+        <v>891.8023236596122</v>
       </c>
       <c r="Q65" t="n">
-        <v>121.1944789010821</v>
+        <v>121.1944673978549</v>
       </c>
       <c r="R65" t="n">
-        <v>669.5665557913425</v>
+        <v>669.5666374540945</v>
       </c>
     </row>
     <row r="66">
@@ -3996,22 +3996,22 @@
         <v>2.8</v>
       </c>
       <c r="M66" t="n">
-        <v>101.9464299041912</v>
+        <v>101.9464260691198</v>
       </c>
       <c r="N66" t="n">
-        <v>104.9790293331269</v>
+        <v>104.9790270042161</v>
       </c>
       <c r="O66" t="n">
-        <v>152.5572498383268</v>
+        <v>152.5572373314974</v>
       </c>
       <c r="P66" t="n">
-        <v>945.5799362058</v>
+        <v>945.5802888567541</v>
       </c>
       <c r="Q66" t="n">
-        <v>142.2390127226727</v>
+        <v>142.2389906840362</v>
       </c>
       <c r="R66" t="n">
-        <v>894.9829619822888</v>
+        <v>894.9831657704783</v>
       </c>
     </row>
     <row r="67">
@@ -4052,22 +4052,22 @@
         <v>2.86</v>
       </c>
       <c r="M67" t="n">
-        <v>104.3474278685397</v>
+        <v>104.3474257034366</v>
       </c>
       <c r="N67" t="n">
-        <v>103.3505960136513</v>
+        <v>103.3505952805919</v>
       </c>
       <c r="O67" t="n">
-        <v>156.1966588365513</v>
+        <v>156.196650454587</v>
       </c>
       <c r="P67" t="n">
-        <v>1025.492314513675</v>
+        <v>1025.49271106536</v>
       </c>
       <c r="Q67" t="n">
-        <v>131.1350826211449</v>
+        <v>131.135065826541</v>
       </c>
       <c r="R67" t="n">
-        <v>1086.872607350888</v>
+        <v>1086.872658396869</v>
       </c>
     </row>
     <row r="68">
@@ -4108,22 +4108,22 @@
         <v>2.55</v>
       </c>
       <c r="M68" s="3" t="n">
-        <v>106.5134710375964</v>
+        <v>106.5134692276869</v>
       </c>
       <c r="N68" s="3" t="n">
-        <v>109.4835644868736</v>
+        <v>109.4835590636833</v>
       </c>
       <c r="O68" s="3" t="n">
-        <v>154.0140903824953</v>
+        <v>154.0140857427668</v>
       </c>
       <c r="P68" s="3" t="n">
-        <v>1369.519696446954</v>
+        <v>1369.520182923256</v>
       </c>
       <c r="Q68" s="3" t="n">
-        <v>132.9471918091454</v>
+        <v>132.947182530961</v>
       </c>
       <c r="R68" s="3" t="n">
-        <v>1437.456952473097</v>
+        <v>1437.457312791659</v>
       </c>
     </row>
     <row r="69">
@@ -4164,22 +4164,22 @@
         <v>2.6</v>
       </c>
       <c r="M69" s="3" t="n">
-        <v>100.8568794478521</v>
+        <v>100.8568654673158</v>
       </c>
       <c r="N69" s="3" t="n">
-        <v>106.644249630433</v>
+        <v>106.6442544409175</v>
       </c>
       <c r="O69" s="3" t="n">
-        <v>157.8706633056499</v>
+        <v>157.8706692190119</v>
       </c>
       <c r="P69" s="3" t="n">
-        <v>1432.372003574803</v>
+        <v>1432.372483137599</v>
       </c>
       <c r="Q69" s="3" t="n">
-        <v>125.1881324044122</v>
+        <v>125.1881263308945</v>
       </c>
       <c r="R69" s="3" t="n">
-        <v>1518.658006783828</v>
+        <v>1518.658692006362</v>
       </c>
     </row>
     <row r="70">
@@ -4220,22 +4220,22 @@
         <v>2.67</v>
       </c>
       <c r="M70" t="n">
-        <v>96.65414390139654</v>
+        <v>96.65414005795267</v>
       </c>
       <c r="N70" t="n">
-        <v>106.8964797504817</v>
+        <v>106.8964805991708</v>
       </c>
       <c r="O70" t="n">
-        <v>155.2863590075499</v>
+        <v>155.2863456955157</v>
       </c>
       <c r="P70" t="n">
-        <v>1427.78745133993</v>
+        <v>1427.787947590759</v>
       </c>
       <c r="Q70" t="n">
-        <v>126.6162547484094</v>
+        <v>126.6162505303238</v>
       </c>
       <c r="R70" t="n">
-        <v>1485.445619752432</v>
+        <v>1485.445896824275</v>
       </c>
     </row>
     <row r="71">
@@ -4276,22 +4276,22 @@
         <v>2.62</v>
       </c>
       <c r="M71" t="n">
-        <v>93.06512399114084</v>
+        <v>93.06512352714147</v>
       </c>
       <c r="N71" t="n">
-        <v>101.8015111869246</v>
+        <v>101.8015107702597</v>
       </c>
       <c r="O71" t="n">
-        <v>146.2495496293114</v>
+        <v>146.2495275766464</v>
       </c>
       <c r="P71" t="n">
-        <v>1542.611460848904</v>
+        <v>1542.611724547781</v>
       </c>
       <c r="Q71" t="n">
-        <v>121.2082237843254</v>
+        <v>121.2082214281356</v>
       </c>
       <c r="R71" t="n">
-        <v>1570.877688754843</v>
+        <v>1570.877965792447</v>
       </c>
     </row>
     <row r="72">
@@ -4332,22 +4332,22 @@
         <v>2.75</v>
       </c>
       <c r="M72" t="n">
-        <v>109.0474208060105</v>
+        <v>109.0474061271542</v>
       </c>
       <c r="N72" t="n">
-        <v>106.6990090773952</v>
+        <v>106.6989993915202</v>
       </c>
       <c r="O72" t="n">
-        <v>150.1763346573113</v>
+        <v>150.1763164341159</v>
       </c>
       <c r="P72" t="n">
-        <v>1570.257835867472</v>
+        <v>1570.258243922381</v>
       </c>
       <c r="Q72" t="n">
-        <v>140.307336218519</v>
+        <v>140.307324945927</v>
       </c>
       <c r="R72" t="n">
-        <v>1624.445528456943</v>
+        <v>1624.445825661683</v>
       </c>
     </row>
     <row r="73">
@@ -4388,22 +4388,22 @@
         <v>2.65</v>
       </c>
       <c r="M73" t="n">
-        <v>125.7098695312202</v>
+        <v>125.7098559914967</v>
       </c>
       <c r="N73" t="n">
-        <v>107.6992388493139</v>
+        <v>107.6992555504447</v>
       </c>
       <c r="O73" t="n">
-        <v>148.0565441686029</v>
+        <v>148.0565108969866</v>
       </c>
       <c r="P73" t="n">
-        <v>1623.65277074529</v>
+        <v>1623.653286321298</v>
       </c>
       <c r="Q73" t="n">
-        <v>147.2911021520394</v>
+        <v>147.2911067875705</v>
       </c>
       <c r="R73" t="n">
-        <v>1678.677683899155</v>
+        <v>1678.6779916422</v>
       </c>
     </row>
     <row r="74">
@@ -4444,22 +4444,22 @@
         <v>2.7</v>
       </c>
       <c r="M74" t="n">
-        <v>118.6266821484177</v>
+        <v>118.6266657810648</v>
       </c>
       <c r="N74" t="n">
-        <v>104.8459876948321</v>
+        <v>104.8459897799837</v>
       </c>
       <c r="O74" t="n">
-        <v>144.7054428288151</v>
+        <v>144.705423382137</v>
       </c>
       <c r="P74" t="n">
-        <v>1990.635771573252</v>
+        <v>1990.636488033048</v>
       </c>
       <c r="Q74" t="n">
-        <v>134.9004203038463</v>
+        <v>134.9004174289825</v>
       </c>
       <c r="R74" t="n">
-        <v>1732.326280833473</v>
+        <v>1732.326695848922</v>
       </c>
     </row>
     <row r="75">
@@ -4500,22 +4500,22 @@
         <v>3.08</v>
       </c>
       <c r="M75" t="n">
-        <v>124.382876298062</v>
+        <v>124.3828682647533</v>
       </c>
       <c r="N75" t="n">
-        <v>106.6853165319505</v>
+        <v>106.6853113858976</v>
       </c>
       <c r="O75" t="n">
-        <v>147.6796999821117</v>
+        <v>147.6796498156545</v>
       </c>
       <c r="P75" t="n">
-        <v>2138.412903424495</v>
+        <v>2138.413482829195</v>
       </c>
       <c r="Q75" t="n">
-        <v>142.309922540387</v>
+        <v>142.3099284798053</v>
       </c>
       <c r="R75" t="n">
-        <v>1689.240829417542</v>
+        <v>1689.241415901625</v>
       </c>
     </row>
     <row r="76">
@@ -4556,22 +4556,22 @@
         <v>3.24</v>
       </c>
       <c r="M76" t="n">
-        <v>127.7719617829249</v>
+        <v>127.7719544961434</v>
       </c>
       <c r="N76" t="n">
-        <v>103.6075644057491</v>
+        <v>103.6075579207537</v>
       </c>
       <c r="O76" t="n">
-        <v>149.2602355793613</v>
+        <v>149.2602324496376</v>
       </c>
       <c r="P76" t="n">
-        <v>1975.662212203988</v>
+        <v>1975.662735012843</v>
       </c>
       <c r="Q76" t="n">
-        <v>146.6408244278952</v>
+        <v>146.6408425913201</v>
       </c>
       <c r="R76" t="n">
-        <v>1631.55076359301</v>
+        <v>1631.551092475338</v>
       </c>
     </row>
     <row r="77">
@@ -4612,22 +4612,22 @@
         <v>3.11</v>
       </c>
       <c r="M77" t="n">
-        <v>125.2158113933079</v>
+        <v>125.2157924435858</v>
       </c>
       <c r="N77" t="n">
-        <v>101.113269063437</v>
+        <v>101.1132741029564</v>
       </c>
       <c r="O77" t="n">
-        <v>149.6567250064888</v>
+        <v>149.6567013347409</v>
       </c>
       <c r="P77" t="n">
-        <v>2010.605857517008</v>
+        <v>2010.606301140026</v>
       </c>
       <c r="Q77" t="n">
-        <v>147.4509322677031</v>
+        <v>147.4509375215345</v>
       </c>
       <c r="R77" t="n">
-        <v>1873.306376546423</v>
+        <v>1873.307029744744</v>
       </c>
     </row>
     <row r="78">
@@ -4668,22 +4668,22 @@
         <v>3.23</v>
       </c>
       <c r="M78" t="n">
-        <v>129.0394738127985</v>
+        <v>129.0394691340401</v>
       </c>
       <c r="N78" t="n">
-        <v>101.7027981250686</v>
+        <v>101.7027976743278</v>
       </c>
       <c r="O78" t="n">
-        <v>142.879754623836</v>
+        <v>142.8797286901632</v>
       </c>
       <c r="P78" t="n">
-        <v>1901.291861393248</v>
+        <v>1901.29252772114</v>
       </c>
       <c r="Q78" t="n">
-        <v>144.8917929130654</v>
+        <v>144.8917920758414</v>
       </c>
       <c r="R78" t="n">
-        <v>1796.756609539987</v>
+        <v>1796.757238457163</v>
       </c>
     </row>
     <row r="79">
@@ -4724,22 +4724,22 @@
         <v>3.28</v>
       </c>
       <c r="M79" t="n">
-        <v>130.9031151085435</v>
+        <v>130.9031057293707</v>
       </c>
       <c r="N79" t="n">
-        <v>92.00477565733648</v>
+        <v>92.00478361023052</v>
       </c>
       <c r="O79" t="n">
-        <v>145.2745564342192</v>
+        <v>145.2745232828059</v>
       </c>
       <c r="P79" t="n">
-        <v>1853.514859698696</v>
+        <v>1853.515430259787</v>
       </c>
       <c r="Q79" t="n">
-        <v>142.9890674167098</v>
+        <v>142.9890759021614</v>
       </c>
       <c r="R79" t="n">
-        <v>1578.896663046806</v>
+        <v>1578.897128919345</v>
       </c>
     </row>
     <row r="80">
@@ -4780,22 +4780,22 @@
         <v>3.17</v>
       </c>
       <c r="M80" t="n">
-        <v>127.5033937344463</v>
+        <v>127.503385962521</v>
       </c>
       <c r="N80" t="n">
-        <v>84.13027766606561</v>
+        <v>84.13026946447994</v>
       </c>
       <c r="O80" t="n">
-        <v>143.5885002800826</v>
+        <v>143.5884932477945</v>
       </c>
       <c r="P80" t="n">
-        <v>2143.397079522749</v>
+        <v>2143.398125756555</v>
       </c>
       <c r="Q80" t="n">
-        <v>141.6220294940447</v>
+        <v>141.6220312034214</v>
       </c>
       <c r="R80" t="n">
-        <v>1552.024109289585</v>
+        <v>1552.024380529356</v>
       </c>
     </row>
     <row r="81">
@@ -4836,22 +4836,22 @@
         <v>3.19</v>
       </c>
       <c r="M81" s="3" t="n">
-        <v>136.0921932443209</v>
+        <v>136.0921752528854</v>
       </c>
       <c r="N81" s="3" t="n">
-        <v>97.41067025957099</v>
+        <v>97.41067256009983</v>
       </c>
       <c r="O81" s="3" t="n">
-        <v>147.1370343027404</v>
+        <v>147.1370272079248</v>
       </c>
       <c r="P81" s="3" t="n">
-        <v>2199.752249890296</v>
+        <v>2199.753013519288</v>
       </c>
       <c r="Q81" s="3" t="n">
-        <v>152.0642289470919</v>
+        <v>152.0642249553502</v>
       </c>
       <c r="R81" s="3" t="n">
-        <v>1649.043784975109</v>
+        <v>1649.044066610918</v>
       </c>
     </row>
     <row r="82">
@@ -4892,22 +4892,22 @@
         <v>3.37</v>
       </c>
       <c r="M82" t="n">
-        <v>135.1540164374827</v>
+        <v>135.1539914419436</v>
       </c>
       <c r="N82" t="n">
-        <v>89.70233721011162</v>
+        <v>89.70233743387915</v>
       </c>
       <c r="O82" t="n">
-        <v>144.0130355561347</v>
+        <v>144.0130166859808</v>
       </c>
       <c r="P82" t="n">
-        <v>2360.045322438538</v>
+        <v>2360.046258841667</v>
       </c>
       <c r="Q82" t="n">
-        <v>154.7132249048571</v>
+        <v>154.7132281407453</v>
       </c>
       <c r="R82" t="n">
-        <v>1450.169651810192</v>
+        <v>1450.170032265938</v>
       </c>
     </row>
     <row r="83">
@@ -4948,22 +4948,22 @@
         <v>3.58</v>
       </c>
       <c r="M83" t="n">
-        <v>140.3524131572027</v>
+        <v>140.3524053379632</v>
       </c>
       <c r="N83" t="n">
-        <v>97.44536207787236</v>
+        <v>97.44535631534666</v>
       </c>
       <c r="O83" t="n">
-        <v>148.1642117502379</v>
+        <v>148.1641863680547</v>
       </c>
       <c r="P83" t="n">
-        <v>2430.505640684879</v>
+        <v>2430.506272596513</v>
       </c>
       <c r="Q83" t="n">
-        <v>157.7723840540678</v>
+        <v>157.7723797804005</v>
       </c>
       <c r="R83" t="n">
-        <v>1402.267713216834</v>
+        <v>1402.267960622868</v>
       </c>
     </row>
     <row r="84">
@@ -5004,22 +5004,22 @@
         <v>3.51</v>
       </c>
       <c r="M84" t="n">
-        <v>137.0036555230053</v>
+        <v>137.0036277819553</v>
       </c>
       <c r="N84" t="n">
-        <v>91.90437262853007</v>
+        <v>91.90437612571735</v>
       </c>
       <c r="O84" t="n">
-        <v>144.5732155959692</v>
+        <v>144.5731893052734</v>
       </c>
       <c r="P84" t="n">
-        <v>2521.895874307743</v>
+        <v>2521.896737379279</v>
       </c>
       <c r="Q84" t="n">
-        <v>155.8181847140169</v>
+        <v>155.818194790208</v>
       </c>
       <c r="R84" t="n">
-        <v>1449.937055712382</v>
+        <v>1449.937387109367</v>
       </c>
     </row>
     <row r="85">
@@ -5060,22 +5060,22 @@
         <v>3.6</v>
       </c>
       <c r="M85" t="n">
-        <v>143.815579334656</v>
+        <v>143.8155597518324</v>
       </c>
       <c r="N85" t="n">
-        <v>94.15387467830529</v>
+        <v>94.15386987235217</v>
       </c>
       <c r="O85" t="n">
-        <v>144.7392536243725</v>
+        <v>144.7392360699459</v>
       </c>
       <c r="P85" t="n">
-        <v>2524.528319090362</v>
+        <v>2524.528922208436</v>
       </c>
       <c r="Q85" t="n">
-        <v>165.7910959643777</v>
+        <v>165.7911047538583</v>
       </c>
       <c r="R85" t="n">
-        <v>1431.853253334769</v>
+        <v>1431.853444663133</v>
       </c>
     </row>
     <row r="86">
@@ -5116,22 +5116,22 @@
         <v>3.68</v>
       </c>
       <c r="M86" t="n">
-        <v>142.0357013421127</v>
+        <v>142.0356848761494</v>
       </c>
       <c r="N86" t="n">
-        <v>92.57399788988351</v>
+        <v>92.57399445457388</v>
       </c>
       <c r="O86" t="n">
-        <v>139.7658092098308</v>
+        <v>139.765782716316</v>
       </c>
       <c r="P86" t="n">
-        <v>2056.304786886275</v>
+        <v>2056.305667523419</v>
       </c>
       <c r="Q86" t="n">
-        <v>159.2857121269633</v>
+        <v>159.2857087054996</v>
       </c>
       <c r="R86" t="n">
-        <v>1343.500833172498</v>
+        <v>1343.501077217149</v>
       </c>
     </row>
     <row r="87">
@@ -5172,22 +5172,22 @@
         <v>3.67</v>
       </c>
       <c r="M87" t="n">
-        <v>152.1997348894887</v>
+        <v>152.1997249681246</v>
       </c>
       <c r="N87" t="n">
-        <v>118.7453882383138</v>
+        <v>118.7453939250492</v>
       </c>
       <c r="O87" t="n">
-        <v>139.6934311647145</v>
+        <v>139.6934056374245</v>
       </c>
       <c r="P87" t="n">
-        <v>1917.442699106247</v>
+        <v>1917.443309347392</v>
       </c>
       <c r="Q87" t="n">
-        <v>170.3776583588561</v>
+        <v>170.3776678536209</v>
       </c>
       <c r="R87" t="n">
-        <v>1391.265589376031</v>
+        <v>1391.265739748291</v>
       </c>
     </row>
     <row r="88">
@@ -5228,22 +5228,22 @@
         <v>3.85</v>
       </c>
       <c r="M88" t="n">
-        <v>156.2847801586474</v>
+        <v>156.2847697768419</v>
       </c>
       <c r="N88" t="n">
-        <v>114.4358256239133</v>
+        <v>114.4358123072375</v>
       </c>
       <c r="O88" t="n">
-        <v>144.166075128864</v>
+        <v>144.1660577276409</v>
       </c>
       <c r="P88" t="n">
-        <v>2005.957706687022</v>
+        <v>2005.958425431494</v>
       </c>
       <c r="Q88" t="n">
-        <v>168.673429762324</v>
+        <v>168.673436061376</v>
       </c>
       <c r="R88" t="n">
-        <v>1292.435560677639</v>
+        <v>1292.435893061061</v>
       </c>
     </row>
     <row r="89">
@@ -5284,22 +5284,22 @@
         <v>4.38</v>
       </c>
       <c r="M89" t="n">
-        <v>156.0117153472004</v>
+        <v>156.0117143799631</v>
       </c>
       <c r="N89" t="n">
-        <v>129.114397513857</v>
+        <v>129.1144019895052</v>
       </c>
       <c r="O89" t="n">
-        <v>149.7028777991538</v>
+        <v>149.7028464500386</v>
       </c>
       <c r="P89" t="n">
-        <v>1856.207179371066</v>
+        <v>1856.20774990973</v>
       </c>
       <c r="Q89" t="n">
-        <v>177.1733242199909</v>
+        <v>177.1733126513817</v>
       </c>
       <c r="R89" t="n">
-        <v>1191.189720310922</v>
+        <v>1191.190034183048</v>
       </c>
     </row>
     <row r="90">
@@ -5340,22 +5340,22 @@
         <v>4.17</v>
       </c>
       <c r="M90" t="n">
-        <v>156.1560239692888</v>
+        <v>156.1560156718381</v>
       </c>
       <c r="N90" t="n">
-        <v>118.2834998050078</v>
+        <v>118.2835112999915</v>
       </c>
       <c r="O90" t="n">
-        <v>155.857587445951</v>
+        <v>155.8575694800351</v>
       </c>
       <c r="P90" t="n">
-        <v>1851.614237294901</v>
+        <v>1851.6147214253</v>
       </c>
       <c r="Q90" t="n">
-        <v>180.8854333798031</v>
+        <v>180.8854378689784</v>
       </c>
       <c r="R90" t="n">
-        <v>1048.465467529866</v>
+        <v>1048.465605096166</v>
       </c>
     </row>
     <row r="91">
@@ -5396,22 +5396,22 @@
         <v>4.26</v>
       </c>
       <c r="M91" t="n">
-        <v>147.4006190788975</v>
+        <v>147.4005932945471</v>
       </c>
       <c r="N91" t="n">
-        <v>103.1306696581524</v>
+        <v>103.1306788245896</v>
       </c>
       <c r="O91" t="n">
-        <v>152.6328072489422</v>
+        <v>152.6327915660292</v>
       </c>
       <c r="P91" t="n">
-        <v>1675.867453334951</v>
+        <v>1675.867821612057</v>
       </c>
       <c r="Q91" t="n">
-        <v>167.5301794722416</v>
+        <v>167.5301754596397</v>
       </c>
       <c r="R91" t="n">
-        <v>845.9728550532481</v>
+        <v>845.9729662705197</v>
       </c>
     </row>
     <row r="92">
@@ -5452,22 +5452,22 @@
         <v>3.88</v>
       </c>
       <c r="M92" t="n">
-        <v>154.470721842668</v>
+        <v>154.4707174089193</v>
       </c>
       <c r="N92" t="n">
-        <v>105.5314693122425</v>
+        <v>105.5314663453258</v>
       </c>
       <c r="O92" t="n">
-        <v>155.7340910700041</v>
+        <v>155.7340724047196</v>
       </c>
       <c r="P92" t="n">
-        <v>1903.560744566979</v>
+        <v>1903.561180203848</v>
       </c>
       <c r="Q92" t="n">
-        <v>172.7816843321866</v>
+        <v>172.7816771712098</v>
       </c>
       <c r="R92" t="n">
-        <v>827.1235106062837</v>
+        <v>827.1238366893643</v>
       </c>
     </row>
     <row r="93">
@@ -5508,22 +5508,22 @@
         <v>3.98</v>
       </c>
       <c r="M93" s="3" t="n">
-        <v>157.4945593653339</v>
+        <v>157.4945446568432</v>
       </c>
       <c r="N93" s="3" t="n">
-        <v>110.1823738316121</v>
+        <v>110.1823830248428</v>
       </c>
       <c r="O93" s="3" t="n">
-        <v>155.7363442381577</v>
+        <v>155.7363328379108</v>
       </c>
       <c r="P93" s="3" t="n">
-        <v>1814.667077260901</v>
+        <v>1814.667728853732</v>
       </c>
       <c r="Q93" s="3" t="n">
-        <v>175.9636848882157</v>
+        <v>175.9636985930933</v>
       </c>
       <c r="R93" s="3" t="n">
-        <v>751.7745839516789</v>
+        <v>751.774680366659</v>
       </c>
     </row>
     <row r="94">
@@ -5564,22 +5564,22 @@
         <v>4.41</v>
       </c>
       <c r="M94" t="n">
-        <v>151.2032154630935</v>
+        <v>151.2032175790608</v>
       </c>
       <c r="N94" t="n">
-        <v>100.0466233761695</v>
+        <v>100.0466232436894</v>
       </c>
       <c r="O94" t="n">
-        <v>150.8977265301609</v>
+        <v>150.897708277856</v>
       </c>
       <c r="P94" t="n">
-        <v>1773.935712103634</v>
+        <v>1773.936156256385</v>
       </c>
       <c r="Q94" t="n">
-        <v>164.0738702627486</v>
+        <v>164.0738779530403</v>
       </c>
       <c r="R94" t="n">
-        <v>611.3911921794736</v>
+        <v>611.3913195408352</v>
       </c>
     </row>
     <row r="95">
@@ -5620,22 +5620,22 @@
         <v>4.37</v>
       </c>
       <c r="M95" t="n">
-        <v>157.9446686088924</v>
+        <v>157.944645927172</v>
       </c>
       <c r="N95" t="n">
-        <v>107.0110445798313</v>
+        <v>107.0110486677763</v>
       </c>
       <c r="O95" t="n">
-        <v>150.2864900794106</v>
+        <v>150.286480629819</v>
       </c>
       <c r="P95" t="n">
-        <v>1691.666568070279</v>
+        <v>1691.667386758266</v>
       </c>
       <c r="Q95" t="n">
-        <v>172.9320419881721</v>
+        <v>172.9320475410137</v>
       </c>
       <c r="R95" t="n">
-        <v>717.947874534904</v>
+        <v>717.9480806720017</v>
       </c>
     </row>
     <row r="96">
@@ -5676,22 +5676,22 @@
         <v>4.11</v>
       </c>
       <c r="M96" t="n">
-        <v>161.2597178542937</v>
+        <v>161.2597276613734</v>
       </c>
       <c r="N96" t="n">
-        <v>103.1780504998288</v>
+        <v>103.1780550043311</v>
       </c>
       <c r="O96" t="n">
-        <v>156.5294852465146</v>
+        <v>156.5294561923434</v>
       </c>
       <c r="P96" t="n">
-        <v>1896.299506922046</v>
+        <v>1896.300090005079</v>
       </c>
       <c r="Q96" t="n">
-        <v>177.0279658589253</v>
+        <v>177.027938010687</v>
       </c>
       <c r="R96" t="n">
-        <v>798.4066738396739</v>
+        <v>798.4068724304198</v>
       </c>
     </row>
     <row r="97">
@@ -5732,22 +5732,22 @@
         <v>4.07</v>
       </c>
       <c r="M97" t="n">
-        <v>160.0503080112092</v>
+        <v>160.0503117281062</v>
       </c>
       <c r="N97" t="n">
-        <v>110.9615744194209</v>
+        <v>110.9615835477329</v>
       </c>
       <c r="O97" t="n">
-        <v>157.2009850829335</v>
+        <v>157.2009547602877</v>
       </c>
       <c r="P97" t="n">
-        <v>1917.379824496153</v>
+        <v>1917.380695108568</v>
       </c>
       <c r="Q97" t="n">
-        <v>177.3076662032768</v>
+        <v>177.307674440675</v>
       </c>
       <c r="R97" t="n">
-        <v>822.0040303290432</v>
+        <v>822.0042343554267</v>
       </c>
     </row>
     <row r="98">
@@ -5788,22 +5788,22 @@
         <v>3.8</v>
       </c>
       <c r="M98" t="n">
-        <v>158.8606276817997</v>
+        <v>158.8606029377696</v>
       </c>
       <c r="N98" t="n">
-        <v>104.8328675631146</v>
+        <v>104.832871071772</v>
       </c>
       <c r="O98" t="n">
-        <v>167.4155415154342</v>
+        <v>167.4155147027576</v>
       </c>
       <c r="P98" t="n">
-        <v>1975.639720636575</v>
+        <v>1975.640457835304</v>
       </c>
       <c r="Q98" t="n">
-        <v>171.6034977417887</v>
+        <v>171.6035009193153</v>
       </c>
       <c r="R98" t="n">
-        <v>813.2537286964762</v>
+        <v>813.2539705461365</v>
       </c>
     </row>
     <row r="99">
@@ -5844,22 +5844,22 @@
         <v>3.91</v>
       </c>
       <c r="M99" t="n">
-        <v>156.5803186316409</v>
+        <v>156.5803053440524</v>
       </c>
       <c r="N99" t="n">
-        <v>104.416192909887</v>
+        <v>104.416189430124</v>
       </c>
       <c r="O99" t="n">
-        <v>167.776725940637</v>
+        <v>167.776709069591</v>
       </c>
       <c r="P99" t="n">
-        <v>1921.9465438264</v>
+        <v>1921.947154911697</v>
       </c>
       <c r="Q99" t="n">
-        <v>160.8391301197269</v>
+        <v>160.8391240427291</v>
       </c>
       <c r="R99" t="n">
-        <v>775.885386905401</v>
+        <v>775.8855804551943</v>
       </c>
     </row>
     <row r="100">
@@ -5900,22 +5900,22 @@
         <v>3.91</v>
       </c>
       <c r="M100" t="n">
-        <v>154.4604666859172</v>
+        <v>154.4604585321645</v>
       </c>
       <c r="N100" t="n">
-        <v>105.1575131715172</v>
+        <v>105.1575105913113</v>
       </c>
       <c r="O100" t="n">
-        <v>170.119997287636</v>
+        <v>170.1199831061443</v>
       </c>
       <c r="P100" t="n">
-        <v>1928.227139925913</v>
+        <v>1928.227933033479</v>
       </c>
       <c r="Q100" t="n">
-        <v>163.5448124430422</v>
+        <v>163.5448020998727</v>
       </c>
       <c r="R100" t="n">
-        <v>850.283210333567</v>
+        <v>850.2833448301136</v>
       </c>
     </row>
     <row r="101">
@@ -5956,22 +5956,22 @@
         <v>3.73</v>
       </c>
       <c r="M101" t="n">
-        <v>151.1413832092609</v>
+        <v>151.1413688103023</v>
       </c>
       <c r="N101" t="n">
-        <v>107.0643160379958</v>
+        <v>107.0643080172437</v>
       </c>
       <c r="O101" t="n">
-        <v>172.3313850174074</v>
+        <v>172.3313565043006</v>
       </c>
       <c r="P101" t="n">
-        <v>1871.123418959458</v>
+        <v>1871.124012716082</v>
       </c>
       <c r="Q101" t="n">
-        <v>168.3876259930509</v>
+        <v>168.387588707094</v>
       </c>
       <c r="R101" t="n">
-        <v>895.4033520517626</v>
+        <v>895.4035451051656</v>
       </c>
     </row>
     <row r="102">
@@ -6012,22 +6012,22 @@
         <v>3.7</v>
       </c>
       <c r="M102" t="n">
-        <v>147.678660787425</v>
+        <v>147.6786385003953</v>
       </c>
       <c r="N102" t="n">
-        <v>104.4072389685124</v>
+        <v>104.4072317264568</v>
       </c>
       <c r="O102" t="n">
-        <v>167.3141116871942</v>
+        <v>167.3140789629893</v>
       </c>
       <c r="P102" t="n">
-        <v>1931.983535681968</v>
+        <v>1931.984124667843</v>
       </c>
       <c r="Q102" t="n">
-        <v>160.0635239273248</v>
+        <v>160.0635290256845</v>
       </c>
       <c r="R102" t="n">
-        <v>919.1693157986236</v>
+        <v>919.1695578825424</v>
       </c>
     </row>
     <row r="103">
@@ -6068,22 +6068,22 @@
         <v>3.85</v>
       </c>
       <c r="M103" t="n">
-        <v>150.5253963854762</v>
+        <v>150.5253891380518</v>
       </c>
       <c r="N103" t="n">
-        <v>106.091413403699</v>
+        <v>106.0914140016929</v>
       </c>
       <c r="O103" t="n">
-        <v>169.4970830960222</v>
+        <v>169.4970592034264</v>
       </c>
       <c r="P103" t="n">
-        <v>2024.134073496189</v>
+        <v>2024.134883944762</v>
       </c>
       <c r="Q103" t="n">
-        <v>159.0154973547809</v>
+        <v>159.015485437679</v>
       </c>
       <c r="R103" t="n">
-        <v>787.4312290160826</v>
+        <v>787.4314767818655</v>
       </c>
     </row>
     <row r="104">
@@ -6124,22 +6124,22 @@
         <v>3.84</v>
       </c>
       <c r="M104" t="n">
-        <v>161.8181353177715</v>
+        <v>161.8181180458683</v>
       </c>
       <c r="N104" t="n">
-        <v>116.2393481688526</v>
+        <v>116.2393646140737</v>
       </c>
       <c r="O104" t="n">
-        <v>165.8750237529238</v>
+        <v>165.8750196369966</v>
       </c>
       <c r="P104" t="n">
-        <v>2104.135150326888</v>
+        <v>2104.136078617876</v>
       </c>
       <c r="Q104" t="n">
-        <v>170.3049069280975</v>
+        <v>170.3048973171494</v>
       </c>
       <c r="R104" t="n">
-        <v>870.6467334748124</v>
+        <v>870.6468824581668</v>
       </c>
     </row>
     <row r="105">
@@ -6180,22 +6180,22 @@
         <v>3.84</v>
       </c>
       <c r="M105" s="3" t="n">
-        <v>163.9460213519798</v>
+        <v>163.9460266345995</v>
       </c>
       <c r="N105" s="3" t="n">
-        <v>110.6407541748721</v>
+        <v>110.6407559477275</v>
       </c>
       <c r="O105" s="3" t="n">
-        <v>166.6150576463907</v>
+        <v>166.6150386349272</v>
       </c>
       <c r="P105" s="3" t="n">
-        <v>2166.050340130452</v>
+        <v>2166.051119134786</v>
       </c>
       <c r="Q105" s="3" t="n">
-        <v>169.9825811951376</v>
+        <v>169.982571640477</v>
       </c>
       <c r="R105" s="3" t="n">
-        <v>779.5725012698099</v>
+        <v>779.5727539685746</v>
       </c>
     </row>
     <row r="106">
@@ -6236,22 +6236,22 @@
         <v>3.97</v>
       </c>
       <c r="M106" t="n">
-        <v>162.435116871098</v>
+        <v>162.4351118001</v>
       </c>
       <c r="N106" t="n">
-        <v>109.9229660409206</v>
+        <v>109.9229558423184</v>
       </c>
       <c r="O106" t="n">
-        <v>168.061344847627</v>
+        <v>168.0613154536782</v>
       </c>
       <c r="P106" t="n">
-        <v>2028.276840504631</v>
+        <v>2028.277611401438</v>
       </c>
       <c r="Q106" t="n">
-        <v>171.8372204765683</v>
+        <v>171.8372102500275</v>
       </c>
       <c r="R106" t="n">
-        <v>776.0768090795328</v>
+        <v>776.0769780209766</v>
       </c>
     </row>
     <row r="107">
@@ -6292,22 +6292,22 @@
         <v>4.11</v>
       </c>
       <c r="M107" t="n">
-        <v>167.980857318355</v>
+        <v>167.9808528552626</v>
       </c>
       <c r="N107" t="n">
-        <v>111.003419090059</v>
+        <v>111.003417858458</v>
       </c>
       <c r="O107" t="n">
-        <v>171.3636296529971</v>
+        <v>171.3636191457917</v>
       </c>
       <c r="P107" t="n">
-        <v>1972.414841504646</v>
+        <v>1972.415589191406</v>
       </c>
       <c r="Q107" t="n">
-        <v>175.5913101847653</v>
+        <v>175.5912920595035</v>
       </c>
       <c r="R107" t="n">
-        <v>767.9704498557242</v>
+        <v>767.9707774396338</v>
       </c>
     </row>
     <row r="108">
@@ -6348,22 +6348,22 @@
         <v>3.81</v>
       </c>
       <c r="M108" t="n">
-        <v>168.6216071205623</v>
+        <v>168.6215924336854</v>
       </c>
       <c r="N108" t="n">
-        <v>113.4489546163955</v>
+        <v>113.4489483571579</v>
       </c>
       <c r="O108" t="n">
-        <v>174.7788396205191</v>
+        <v>174.7788249727197</v>
       </c>
       <c r="P108" t="n">
-        <v>2001.507735080219</v>
+        <v>2001.508371927525</v>
       </c>
       <c r="Q108" t="n">
-        <v>172.1349204299516</v>
+        <v>172.1349216255006</v>
       </c>
       <c r="R108" t="n">
-        <v>803.6981124025461</v>
+        <v>803.698328822361</v>
       </c>
     </row>
     <row r="109">
@@ -6404,22 +6404,22 @@
         <v>3.74</v>
       </c>
       <c r="M109" t="n">
-        <v>170.3033443398824</v>
+        <v>170.3033330623022</v>
       </c>
       <c r="N109" t="n">
-        <v>112.5852258999318</v>
+        <v>112.585223746124</v>
       </c>
       <c r="O109" t="n">
-        <v>176.6482545004284</v>
+        <v>176.6482347824997</v>
       </c>
       <c r="P109" t="n">
-        <v>2069.770013226697</v>
+        <v>2069.770784798596</v>
       </c>
       <c r="Q109" t="n">
-        <v>173.4922529196261</v>
+        <v>173.4922474255485</v>
       </c>
       <c r="R109" t="n">
-        <v>851.8265557510906</v>
+        <v>851.8267788061371</v>
       </c>
     </row>
     <row r="110">
@@ -6460,22 +6460,22 @@
         <v>3.79</v>
       </c>
       <c r="M110" t="n">
-        <v>177.6777794739595</v>
+        <v>177.677753843991</v>
       </c>
       <c r="N110" t="n">
-        <v>114.2459929682231</v>
+        <v>114.2459989282934</v>
       </c>
       <c r="O110" t="n">
-        <v>181.9816416343741</v>
+        <v>181.9816168979239</v>
       </c>
       <c r="P110" t="n">
-        <v>2122.079955272615</v>
+        <v>2122.080634048682</v>
       </c>
       <c r="Q110" t="n">
-        <v>170.1439107400517</v>
+        <v>170.1439426792902</v>
       </c>
       <c r="R110" t="n">
-        <v>860.6893487412444</v>
+        <v>860.6895766229879</v>
       </c>
     </row>
     <row r="111">
@@ -6516,22 +6516,22 @@
         <v>3.86</v>
       </c>
       <c r="M111" t="n">
-        <v>181.7235898330149</v>
+        <v>181.7235688439439</v>
       </c>
       <c r="N111" t="n">
-        <v>113.7345535426124</v>
+        <v>113.734545437603</v>
       </c>
       <c r="O111" t="n">
-        <v>185.5366693082331</v>
+        <v>185.536633427889</v>
       </c>
       <c r="P111" t="n">
-        <v>2221.377820554736</v>
+        <v>2221.378534199563</v>
       </c>
       <c r="Q111" t="n">
-        <v>176.7683933073925</v>
+        <v>176.7683887403995</v>
       </c>
       <c r="R111" t="n">
-        <v>796.3757002535972</v>
+        <v>796.3759933570624</v>
       </c>
     </row>
     <row r="112">
@@ -6572,22 +6572,22 @@
         <v>3.85</v>
       </c>
       <c r="M112" t="n">
-        <v>187.7364039543114</v>
+        <v>187.7363919378955</v>
       </c>
       <c r="N112" t="n">
-        <v>114.089560587066</v>
+        <v>114.0895607196094</v>
       </c>
       <c r="O112" t="n">
-        <v>183.7043206067689</v>
+        <v>183.7042899122306</v>
       </c>
       <c r="P112" t="n">
-        <v>2293.226651282825</v>
+        <v>2293.227348939291</v>
       </c>
       <c r="Q112" t="n">
-        <v>171.8898765328798</v>
+        <v>171.8898663783141</v>
       </c>
       <c r="R112" t="n">
-        <v>794.1981486573568</v>
+        <v>794.1983586397096</v>
       </c>
     </row>
     <row r="113">
@@ -6628,22 +6628,22 @@
         <v>3.97</v>
       </c>
       <c r="M113" t="n">
-        <v>186.2415494934475</v>
+        <v>186.2415217383354</v>
       </c>
       <c r="N113" t="n">
-        <v>117.5789807040146</v>
+        <v>117.578978319408</v>
       </c>
       <c r="O113" t="n">
-        <v>191.4531791859021</v>
+        <v>191.4531391431029</v>
       </c>
       <c r="P113" t="n">
-        <v>2264.581772236661</v>
+        <v>2264.582509241456</v>
       </c>
       <c r="Q113" t="n">
-        <v>174.122838816557</v>
+        <v>174.1228216079261</v>
       </c>
       <c r="R113" t="n">
-        <v>897.3611816276569</v>
+        <v>897.3614477648473</v>
       </c>
     </row>
     <row r="114">
@@ -6684,22 +6684,22 @@
         <v>3.89</v>
       </c>
       <c r="M114" t="n">
-        <v>189.3714275395985</v>
+        <v>189.3714065752639</v>
       </c>
       <c r="N114" t="n">
-        <v>109.9133178311146</v>
+        <v>109.9133142809535</v>
       </c>
       <c r="O114" t="n">
-        <v>189.2829106833151</v>
+        <v>189.2828933933023</v>
       </c>
       <c r="P114" t="n">
-        <v>1983.216024153979</v>
+        <v>1983.216797758819</v>
       </c>
       <c r="Q114" t="n">
-        <v>169.1980515278075</v>
+        <v>169.1980530095952</v>
       </c>
       <c r="R114" t="n">
-        <v>1011.977551894753</v>
+        <v>1011.977808091033</v>
       </c>
     </row>
     <row r="115">
@@ -6740,22 +6740,22 @@
         <v>3.86</v>
       </c>
       <c r="M115" t="n">
-        <v>187.9842494883797</v>
+        <v>187.98423364973</v>
       </c>
       <c r="N115" t="n">
-        <v>108.1873438852826</v>
+        <v>108.1873445976669</v>
       </c>
       <c r="O115" t="n">
-        <v>189.8747694463314</v>
+        <v>189.8747522059505</v>
       </c>
       <c r="P115" t="n">
-        <v>2181.568071514296</v>
+        <v>2181.568735352678</v>
       </c>
       <c r="Q115" t="n">
-        <v>158.7202243737491</v>
+        <v>158.7202166271665</v>
       </c>
       <c r="R115" t="n">
-        <v>1054.214158728158</v>
+        <v>1054.21442793061</v>
       </c>
     </row>
     <row r="116">
@@ -6796,22 +6796,22 @@
         <v>3.72</v>
       </c>
       <c r="M116" t="n">
-        <v>198.3642609085469</v>
+        <v>198.3642323225625</v>
       </c>
       <c r="N116" t="n">
-        <v>112.6916370630665</v>
+        <v>112.6916323108251</v>
       </c>
       <c r="O116" t="n">
-        <v>198.1705438671877</v>
+        <v>198.1705198148931</v>
       </c>
       <c r="P116" t="n">
-        <v>2150.625346317037</v>
+        <v>2150.626009102244</v>
       </c>
       <c r="Q116" t="n">
-        <v>156.3990163499795</v>
+        <v>156.3990038247527</v>
       </c>
       <c r="R116" t="n">
-        <v>987.5533071918916</v>
+        <v>987.5535624449169</v>
       </c>
     </row>
     <row r="117">
@@ -6852,22 +6852,22 @@
         <v>3.76</v>
       </c>
       <c r="M117" t="n">
-        <v>218.4672279366905</v>
+        <v>218.4672114301698</v>
       </c>
       <c r="N117" t="n">
-        <v>116.8869263116959</v>
+        <v>116.8869314728614</v>
       </c>
       <c r="O117" t="n">
-        <v>204.1826106372814</v>
+        <v>204.1825968153649</v>
       </c>
       <c r="P117" t="n">
-        <v>1857.218540441219</v>
+        <v>1857.219180597261</v>
       </c>
       <c r="Q117" t="n">
-        <v>167.4863891134006</v>
+        <v>167.4863781923875</v>
       </c>
       <c r="R117" t="n">
-        <v>899.8573284463046</v>
+        <v>899.8576017828602</v>
       </c>
     </row>
     <row r="118">
@@ -6908,22 +6908,22 @@
         <v>3.71</v>
       </c>
       <c r="M118" t="n">
-        <v>217.085016348435</v>
+        <v>217.084985685251</v>
       </c>
       <c r="N118" t="n">
-        <v>114.3875657090406</v>
+        <v>114.387568863797</v>
       </c>
       <c r="O118" t="n">
-        <v>215.1839546206426</v>
+        <v>215.1839174545289</v>
       </c>
       <c r="P118" t="n">
-        <v>1755.430990509585</v>
+        <v>1755.431602677422</v>
       </c>
       <c r="Q118" t="n">
-        <v>157.2847183930647</v>
+        <v>157.284704027436</v>
       </c>
       <c r="R118" t="n">
-        <v>956.5221564784628</v>
+        <v>956.5224439207336</v>
       </c>
     </row>
     <row r="119">
@@ -6964,22 +6964,22 @@
         <v>3.92</v>
       </c>
       <c r="M119" s="3" t="n">
-        <v>214.6197543640977</v>
+        <v>214.6197324629407</v>
       </c>
       <c r="N119" s="3" t="n">
-        <v>114.9497478198026</v>
+        <v>114.9497432653407</v>
       </c>
       <c r="O119" s="3" t="n">
-        <v>217.8415307291696</v>
+        <v>217.8414956246776</v>
       </c>
       <c r="P119" s="3" t="n">
-        <v>1787.641959361786</v>
+        <v>1787.642625541818</v>
       </c>
       <c r="Q119" s="3" t="n">
-        <v>153.5998670377484</v>
+        <v>153.5998677557627</v>
       </c>
       <c r="R119" s="3" t="n">
-        <v>959.4028545253725</v>
+        <v>959.4031005551029</v>
       </c>
     </row>
     <row r="120">
@@ -7020,22 +7020,22 @@
         <v>3.81</v>
       </c>
       <c r="M120" t="n">
-        <v>215.6979788375372</v>
+        <v>215.6979574481733</v>
       </c>
       <c r="N120" t="n">
-        <v>116.1721239407171</v>
+        <v>116.1721184418543</v>
       </c>
       <c r="O120" t="n">
-        <v>220.6866796393185</v>
+        <v>220.6866543595742</v>
       </c>
       <c r="P120" t="n">
-        <v>1797.779163244606</v>
+        <v>1797.779786151261</v>
       </c>
       <c r="Q120" t="n">
-        <v>152.3899876355784</v>
+        <v>152.3899955696756</v>
       </c>
       <c r="R120" t="n">
-        <v>993.3290617022241</v>
+        <v>993.3294278075415</v>
       </c>
     </row>
     <row r="121">
@@ -7076,22 +7076,22 @@
         <v>3.82</v>
       </c>
       <c r="M121" t="n">
-        <v>217.0264815330754</v>
+        <v>217.0264702619863</v>
       </c>
       <c r="N121" t="n">
-        <v>119.9192814649131</v>
+        <v>119.9192798580539</v>
       </c>
       <c r="O121" t="n">
-        <v>225.4302661014434</v>
+        <v>225.430234606078</v>
       </c>
       <c r="P121" t="n">
-        <v>2070.550355007064</v>
+        <v>2070.551041061854</v>
       </c>
       <c r="Q121" t="n">
-        <v>157.984865595238</v>
+        <v>157.9848448702949</v>
       </c>
       <c r="R121" t="n">
-        <v>1097.909703164781</v>
+        <v>1097.910039940701</v>
       </c>
     </row>
     <row r="122">
@@ -7132,22 +7132,22 @@
         <v>3.81</v>
       </c>
       <c r="M122" t="n">
-        <v>212.2118393757991</v>
+        <v>212.2118138083424</v>
       </c>
       <c r="N122" t="n">
-        <v>114.8093943450448</v>
+        <v>114.8093942394136</v>
       </c>
       <c r="O122" t="n">
-        <v>228.1030968256887</v>
+        <v>228.1030596458334</v>
       </c>
       <c r="P122" t="n">
-        <v>1820.976083311235</v>
+        <v>1820.976781622559</v>
       </c>
       <c r="Q122" t="n">
-        <v>152.1773302868199</v>
+        <v>152.1773320696612</v>
       </c>
       <c r="R122" t="n">
-        <v>1040.086284107638</v>
+        <v>1040.086555188728</v>
       </c>
     </row>
     <row r="123">
@@ -7188,22 +7188,22 @@
         <v>3.79</v>
       </c>
       <c r="M123" t="n">
-        <v>216.5930012138706</v>
+        <v>216.5929820536581</v>
       </c>
       <c r="N123" t="n">
-        <v>119.7964578840504</v>
+        <v>119.7964563306469</v>
       </c>
       <c r="O123" t="n">
-        <v>237.6619220296463</v>
+        <v>237.6618745084309</v>
       </c>
       <c r="P123" t="n">
-        <v>1585.432105358776</v>
+        <v>1585.432731975401</v>
       </c>
       <c r="Q123" t="n">
-        <v>141.7103118601667</v>
+        <v>141.7103104240868</v>
       </c>
       <c r="R123" t="n">
-        <v>922.0195421851488</v>
+        <v>922.0197345426138</v>
       </c>
     </row>
     <row r="124">
@@ -7244,22 +7244,22 @@
         <v>3.77</v>
       </c>
       <c r="M124" s="3" t="n">
-        <v>209.1178107862522</v>
+        <v>209.1177919955135</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>116.7757700786058</v>
+        <v>116.7757685470425</v>
       </c>
       <c r="O124" s="3" t="n">
-        <v>236.0877792961903</v>
+        <v>236.0877465189258</v>
       </c>
       <c r="P124" s="3" t="n">
-        <v>1570.898336797052</v>
+        <v>1570.898895362191</v>
       </c>
       <c r="Q124" s="3" t="n">
-        <v>139.0093987390431</v>
+        <v>139.0093969452183</v>
       </c>
       <c r="R124" s="3" t="n">
-        <v>874.2065864780645</v>
+        <v>874.2068538965358</v>
       </c>
     </row>
     <row r="125">
@@ -7300,22 +7300,22 @@
         <v>3.66</v>
       </c>
       <c r="M125" t="n">
-        <v>210.3467234739217</v>
+        <v>210.3466992498875</v>
       </c>
       <c r="N125" t="n">
-        <v>113.6282981849911</v>
+        <v>113.6282924930139</v>
       </c>
       <c r="O125" t="n">
-        <v>244.2690431297513</v>
+        <v>244.269011338987</v>
       </c>
       <c r="P125" t="n">
-        <v>1535.603521560082</v>
+        <v>1535.604031085544</v>
       </c>
       <c r="Q125" t="n">
-        <v>145.5124010855578</v>
+        <v>145.5124108617425</v>
       </c>
       <c r="R125" t="n">
-        <v>902.174699579404</v>
+        <v>902.1749356119599</v>
       </c>
     </row>
     <row r="126">
@@ -7356,22 +7356,22 @@
         <v>3.52</v>
       </c>
       <c r="M126" t="n">
-        <v>204.588868217006</v>
+        <v>204.5888547557031</v>
       </c>
       <c r="N126" t="n">
-        <v>111.5759540192424</v>
+        <v>111.5759485811558</v>
       </c>
       <c r="O126" t="n">
-        <v>252.5168648646359</v>
+        <v>252.516825580797</v>
       </c>
       <c r="P126" t="n">
-        <v>1588.889794023164</v>
+        <v>1588.890252364737</v>
       </c>
       <c r="Q126" t="n">
-        <v>143.6950242380693</v>
+        <v>143.6950189316279</v>
       </c>
       <c r="R126" t="n">
-        <v>878.884802025575</v>
+        <v>878.885075902328</v>
       </c>
     </row>
     <row r="127">
@@ -7412,22 +7412,22 @@
         <v>3.47</v>
       </c>
       <c r="M127" t="n">
-        <v>202.7286958236731</v>
+        <v>202.7286774691023</v>
       </c>
       <c r="N127" t="n">
-        <v>116.7663057972959</v>
+        <v>116.7662997068193</v>
       </c>
       <c r="O127" t="n">
-        <v>263.7674275630359</v>
+        <v>263.7673908463964</v>
       </c>
       <c r="P127" t="n">
-        <v>1702.999801173488</v>
+        <v>1703.000403664495</v>
       </c>
       <c r="Q127" t="n">
-        <v>149.4021688972053</v>
+        <v>149.4021668901691</v>
       </c>
       <c r="R127" t="n">
-        <v>836.9481741044542</v>
+        <v>836.9484741903115</v>
       </c>
     </row>
     <row r="128">
@@ -7468,22 +7468,22 @@
         <v>3.37</v>
       </c>
       <c r="M128" t="n">
-        <v>196.7065672743221</v>
+        <v>196.7065493168377</v>
       </c>
       <c r="N128" t="n">
-        <v>116.4514067861755</v>
+        <v>116.4514049923657</v>
       </c>
       <c r="O128" t="n">
-        <v>275.7312963852951</v>
+        <v>275.7312781685512</v>
       </c>
       <c r="P128" t="n">
-        <v>1799.944906520402</v>
+        <v>1799.945511522417</v>
       </c>
       <c r="Q128" t="n">
-        <v>156.4029323819931</v>
+        <v>156.4029358554356</v>
       </c>
       <c r="R128" t="n">
-        <v>835.8472830673883</v>
+        <v>835.847502367208</v>
       </c>
     </row>
     <row r="129">
@@ -7524,22 +7524,22 @@
         <v>3.39</v>
       </c>
       <c r="M129" t="n">
-        <v>209.8583026088833</v>
+        <v>209.85828338132</v>
       </c>
       <c r="N129" t="n">
-        <v>119.9050457122265</v>
+        <v>119.9050439428864</v>
       </c>
       <c r="O129" t="n">
-        <v>268.6691557501098</v>
+        <v>268.6691278766402</v>
       </c>
       <c r="P129" t="n">
-        <v>1821.888453672412</v>
+        <v>1821.889106651544</v>
       </c>
       <c r="Q129" t="n">
-        <v>164.7329437304167</v>
+        <v>164.7329364771359</v>
       </c>
       <c r="R129" t="n">
-        <v>789.282094767094</v>
+        <v>789.2823709585531</v>
       </c>
     </row>
     <row r="130">
@@ -7580,22 +7580,22 @@
         <v>3.45</v>
       </c>
       <c r="M130" t="n">
-        <v>215.9361663371589</v>
+        <v>215.9361465504395</v>
       </c>
       <c r="N130" t="n">
-        <v>124.6630051844465</v>
+        <v>124.6630033779737</v>
       </c>
       <c r="O130" t="n">
-        <v>274.9331072287118</v>
+        <v>274.9330622738136</v>
       </c>
       <c r="P130" t="n">
-        <v>1799.197055173019</v>
+        <v>1799.197666288034</v>
       </c>
       <c r="Q130" t="n">
-        <v>168.8085616113662</v>
+        <v>168.8085553685743</v>
       </c>
       <c r="R130" t="n">
-        <v>812.6434588287669</v>
+        <v>812.6437049544469</v>
       </c>
     </row>
     <row r="131">
@@ -7636,22 +7636,22 @@
         <v>3.49</v>
       </c>
       <c r="M131" t="n">
-        <v>213.4749004738903</v>
+        <v>213.4748809127023</v>
       </c>
       <c r="N131" t="n">
-        <v>126.3465125275787</v>
+        <v>126.3465107099351</v>
       </c>
       <c r="O131" t="n">
-        <v>273.1133337115353</v>
+        <v>273.1133072706958</v>
       </c>
       <c r="P131" t="n">
-        <v>2135.056009008865</v>
+        <v>2135.05680078673</v>
       </c>
       <c r="Q131" t="n">
-        <v>163.8540334362349</v>
+        <v>163.8540330287217</v>
       </c>
       <c r="R131" t="n">
-        <v>879.2840507898841</v>
+        <v>879.284278047472</v>
       </c>
     </row>
     <row r="132">
@@ -7692,22 +7692,22 @@
         <v>3.47</v>
       </c>
       <c r="M132" t="n">
-        <v>219.4232638227553</v>
+        <v>219.4232437165053</v>
       </c>
       <c r="N132" t="n">
-        <v>124.9059051725063</v>
+        <v>124.9059033755876</v>
       </c>
       <c r="O132" t="n">
-        <v>287.1095107657425</v>
+        <v>287.1094721487543</v>
       </c>
       <c r="P132" t="n">
-        <v>1935.452968870005</v>
+        <v>1935.453631916823</v>
       </c>
       <c r="Q132" t="n">
-        <v>141.2916647312525</v>
+        <v>141.2916699352634</v>
       </c>
       <c r="R132" t="n">
-        <v>883.6800045154627</v>
+        <v>883.6802952796814</v>
       </c>
     </row>
     <row r="133">
@@ -7748,22 +7748,22 @@
         <v>3.49</v>
       </c>
       <c r="M133" t="n">
-        <v>233.3124582722894</v>
+        <v>233.312436893341</v>
       </c>
       <c r="N133" t="n">
-        <v>128.7451893438608</v>
+        <v>128.7451874917095</v>
       </c>
       <c r="O133" t="n">
-        <v>287.6378479848539</v>
+        <v>287.6378085348784</v>
       </c>
       <c r="P133" t="n">
-        <v>1734.404447819877</v>
+        <v>1734.405043687135</v>
       </c>
       <c r="Q133" t="n">
-        <v>154.038939465042</v>
+        <v>154.0389451310591</v>
       </c>
       <c r="R133" t="n">
-        <v>950.8758858370733</v>
+        <v>950.876095230484</v>
       </c>
     </row>
     <row r="134">
@@ -7804,22 +7804,22 @@
         <v>3.5</v>
       </c>
       <c r="M134" t="n">
-        <v>251.875322191347</v>
+        <v>251.8752991114414</v>
       </c>
       <c r="N134" t="n">
-        <v>129.3130847932198</v>
+        <v>129.3130829328987</v>
       </c>
       <c r="O134" t="n">
-        <v>312.5393764578505</v>
+        <v>312.5393331490387</v>
       </c>
       <c r="P134" t="n">
-        <v>1715.301603272256</v>
+        <v>1715.302192576592</v>
       </c>
       <c r="Q134" t="n">
-        <v>152.0508513130379</v>
+        <v>152.0508567752879</v>
       </c>
       <c r="R134" t="n">
-        <v>953.7588385372014</v>
+        <v>953.7591106305374</v>
       </c>
     </row>
     <row r="135">
@@ -7860,22 +7860,22 @@
         <v>3.48</v>
       </c>
       <c r="M135" t="n">
-        <v>248.7708797482085</v>
+        <v>248.7708569527701</v>
       </c>
       <c r="N135" t="n">
-        <v>127.2490323452918</v>
+        <v>127.2490305146644</v>
       </c>
       <c r="O135" t="n">
-        <v>311.1049468362271</v>
+        <v>311.1048947977416</v>
       </c>
       <c r="P135" t="n">
-        <v>1665.419693763954</v>
+        <v>1665.420265930997</v>
       </c>
       <c r="Q135" t="n">
-        <v>149.3331410297488</v>
+        <v>149.3331412001643</v>
       </c>
       <c r="R135" t="n">
-        <v>904.2540631907384</v>
+        <v>904.2542902011654</v>
       </c>
     </row>
     <row r="136">
@@ -7916,22 +7916,22 @@
         <v>3.63</v>
       </c>
       <c r="M136" t="n">
-        <v>241.7000063249476</v>
+        <v>241.6999841774293</v>
       </c>
       <c r="N136" t="n">
-        <v>138.5071545604356</v>
+        <v>138.5071525678469</v>
       </c>
       <c r="O136" t="n">
-        <v>297.9253707722796</v>
+        <v>297.925329919361</v>
       </c>
       <c r="P136" t="n">
-        <v>1571.707312722754</v>
+        <v>1571.707852694228</v>
       </c>
       <c r="Q136" t="n">
-        <v>194.0739009981863</v>
+        <v>194.0739006780349</v>
       </c>
       <c r="R136" t="n">
-        <v>1050.644098101115</v>
+        <v>1050.644362338325</v>
       </c>
     </row>
     <row r="137">
@@ -7972,22 +7972,22 @@
         <v>3.57</v>
       </c>
       <c r="M137" t="n">
-        <v>240.931896698982</v>
+        <v>240.9318746218474</v>
       </c>
       <c r="N137" t="n">
-        <v>140.2206858115785</v>
+        <v>140.2206837943386</v>
       </c>
       <c r="O137" t="n">
-        <v>309.7923406719004</v>
+        <v>309.792298064396</v>
       </c>
       <c r="P137" t="n">
-        <v>2066.955874718228</v>
+        <v>2066.956584835947</v>
       </c>
       <c r="Q137" t="n">
-        <v>188.2776696386924</v>
+        <v>188.2776693281026</v>
       </c>
       <c r="R137" t="n">
-        <v>1126.118702336489</v>
+        <v>1126.118985555578</v>
       </c>
     </row>
     <row r="138">
@@ -8028,22 +8028,22 @@
         <v>3.56</v>
       </c>
       <c r="M138" t="n">
-        <v>236.4405919837912</v>
+        <v>236.440570318205</v>
       </c>
       <c r="N138" t="n">
-        <v>132.5133146376059</v>
+        <v>132.5133127312455</v>
       </c>
       <c r="O138" t="n">
-        <v>297.0924036216358</v>
+        <v>297.0923627608261</v>
       </c>
       <c r="P138" t="n">
-        <v>2483.468236844959</v>
+        <v>2483.469090058528</v>
       </c>
       <c r="Q138" t="n">
-        <v>171.3966893562857</v>
+        <v>171.3966890735434</v>
       </c>
       <c r="R138" t="n">
-        <v>1215.376844947501</v>
+        <v>1215.377150615032</v>
       </c>
     </row>
     <row r="139">
@@ -8084,22 +8084,22 @@
         <v>3.6</v>
       </c>
       <c r="M139" t="n">
-        <v>238.3308378312827</v>
+        <v>238.330815992489</v>
       </c>
       <c r="N139" t="n">
-        <v>138.2781594633694</v>
+        <v>138.2781574740749</v>
       </c>
       <c r="O139" t="n">
-        <v>296.0762224982038</v>
+        <v>296.0761817771554</v>
       </c>
       <c r="P139" t="n">
-        <v>2590.2654316661</v>
+        <v>2590.266321570622</v>
       </c>
       <c r="Q139" t="n">
-        <v>164.2862588247784</v>
+        <v>164.2862585537657</v>
       </c>
       <c r="R139" t="n">
-        <v>1039.541903918486</v>
+        <v>1039.542165363492</v>
       </c>
     </row>
     <row r="140">
@@ -8140,22 +8140,22 @@
         <v>3.7</v>
       </c>
       <c r="M140" t="n">
-        <v>250.4626586625073</v>
+        <v>250.4626357120475</v>
       </c>
       <c r="N140" t="n">
-        <v>145.2305281030831</v>
+        <v>145.2305260137706</v>
       </c>
       <c r="O140" t="n">
-        <v>294.3227513039615</v>
+        <v>294.3227108240779</v>
       </c>
       <c r="P140" t="n">
-        <v>2723.765295899652</v>
+        <v>2723.766231669023</v>
       </c>
       <c r="Q140" t="n">
-        <v>176.1758557479156</v>
+        <v>176.1758554572894</v>
       </c>
       <c r="R140" t="n">
-        <v>1043.998125686649</v>
+        <v>1043.998388252396</v>
       </c>
     </row>
     <row r="141">
@@ -8196,22 +8196,22 @@
         <v>3.8</v>
       </c>
       <c r="M141" t="n">
-        <v>247.4756342952685</v>
+        <v>247.4756116185166</v>
       </c>
       <c r="N141" t="n">
-        <v>152.1903980384033</v>
+        <v>152.1903958489648</v>
       </c>
       <c r="O141" t="n">
-        <v>297.6635873632664</v>
+        <v>297.6635464238987</v>
       </c>
       <c r="P141" t="n">
-        <v>2759.293709065365</v>
+        <v>2759.294657040779</v>
       </c>
       <c r="Q141" t="n">
-        <v>172.5598040000645</v>
+        <v>172.5598037154035</v>
       </c>
       <c r="R141" t="n">
-        <v>1039.975059565733</v>
+        <v>1039.975321119678</v>
       </c>
     </row>
   </sheetData>

</xml_diff>